<commit_message>
Follow tflspec's tfl_ prefix
tflspec 0.0.9 gives every export the tfl_ prefix (ichirio/tflspec#9)
and keeps the former names as aliases.  tflplanner now calls tflspec
by the new names, and the programs it writes and the app's hints use
them: tfl_ard_normalize(), tfl_read_report_spec(), tfl_plan(),
tfl_report(), tfl_report_path().  The ARD definition object it builds
takes tflspec's class name tfl_ard_spec.  Requires tflspec >= 0.0.9.

The sample study's workbooks are regenerated (rework code and the
_README text: names only).  Checked on the sample study against the
code before the change: all 16 RTF identical and the ARD equal; the
programs differ only by the function names (and so their checksums).
The old tflplanner also runs unchanged on the new tflspec (all 38
programs and 16 RTF identical).

Closes #11

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -400,7 +400,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>rtfreporter の表の定義ファイル（table spec）（spec_version 1）。rtf_plan(data; spec = read_table_spec(path; output_id = )) で読む。名前が _ で始まるシートは読まれない（このシート）。</t>
+          <t>rtfreporter の表の定義ファイル（table spec）（spec_version 1）。tfl_plan(data; spec = tfl_read_table_spec(path; output_id = )) で読む。名前が _ で始まるシートは読まれない（このシート）。</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。rtf_plan(data; spec = read_table_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
+          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。tfl_plan(data; spec = tfl_read_table_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>plan_paginate_rows() の max_rows / split / by / min_group_rows / cont_label。先頭・末尾の空白を残すときは引用符で囲む。</t>
+          <t>tfl_plan_paginate_rows() の max_rows / split / by / min_group_rows / cont_label。先頭・末尾の空白を残すときは引用符で囲む。</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>plan_row_group() の col / mode / collapse。collapse は TRUE か列（名前・位置）の | 区切り。</t>
+          <t>tfl_plan_row_group() の col / mode / collapse。collapse は TRUE か列（名前・位置）の | 区切り。</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>group_page = TRUE で group_col の値ごとに改ページ（plan_paginate_group）。group_show = FALSE でその列を表示しない。</t>
+          <t>group_page = TRUE で group_col の値ごとに改ページ（tfl_plan_paginate_group）。group_show = FALSE でその列を表示しない。</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>plan_blanks() の where / first / last / counted。</t>
+          <t>tfl_plan_blanks() の where / first / last / counted。</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>plan_stub() の vars / into / indent / group_summary / before。</t>
+          <t>tfl_plan_stub() の vars / into / indent / group_summary / before。</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>plan_paginate_cols() の every / at / carry / order（列方向のページ分割）。</t>
+          <t>tfl_plan_paginate_cols() の every / at / carry / order（列方向のページ分割）。</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>以下は表の周りの定義。read_report_spec(c(report.xlsx; tables.xlsx); output_id = ) で 1 冊でも分冊でも読める。同じシートに行があるのは 1 冊だけにする（空のシートと study は重なってよい）。rtf_report(spec; plan) で rtf_document、report_path(spec) で出力先。</t>
+          <t>以下は表の周りの定義。tfl_read_report_spec(c(report.xlsx; tables.xlsx); output_id = ) で 1 冊でも分冊でも読める。同じシートに行があるのは 1 冊だけにする（空のシートと study は重なってよい）。tfl_report(spec; plan) で rtf_document、tfl_report_path(spec) で出力先。</t>
         </is>
       </c>
     </row>
@@ -2852,7 +2852,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>data &lt;- ard_normalize(ard, hierarchy = c("AEBODSYS", "AEDECOD"),
+          <t>data &lt;- tfl_ard_normalize(ard, hierarchy = c("AEBODSYS", "AEDECOD"),
                       overall = "Any TEAE")</t>
         </is>
       </c>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>data &lt;- ard_normalize(ard)
+          <t>data &lt;- tfl_ard_normalize(ard)
 # row labels: the median, and the event-free probability by day (day 0 left out)
 is_time &lt;- data$variable == "time"
 data$.label[data$variable == "prob"] &lt;- "Median (95% CI)"

</xml_diff>

<commit_message>
Follow plan E: the table engine is rtfreporter's
tflspec 0.0.23 (feat/e4-spec-only) keeps the specifications only; the ARD
functions and the plan moved to rtfreporter 0.8.0.9087 (feat/491-plan-engine)
as normalize_ard(), table_plan(), plan_*(), plan_apply(), with no aliases.

- builder preview: rtfreporter::plan_apply(); assist: rtfreporter::normalize_ard()
- generated programs and the built-in table_process template write
  normalize_ard(ard); the i18n key (app.R / strings.csv) changed together,
  the stale duplicate key dropped
- saved code is rewritten as it is read (.renamed_calls()): study workbooks'
  _tflplanner sheet, the app's state.json, company standards' code templates
- DESCRIPTION: rtfreporter >= 0.8.0.9087, tflspec >= 0.0.23
- SAMPLE-01 regenerated (13/13 programs run); its 8 RTFs are byte-identical
  to main's on the former engine
- tests, man, NEWS, README, ja-guide install lines, data-raw scripts

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -400,7 +400,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>rtfreporter の表の定義ファイル（table spec）（spec_version 1）。tfl_plan(data; spec = tfl_read_table_spec(path; output_id = )) で読む。名前が _ で始まるシートは読まれない（このシート）。</t>
+          <t>rtfreporter の表の定義ファイル（table spec）（spec_version 1）。tfl_table_plan(data; tfl_read_table_spec(path; output_id = )) で読む。名前が _ で始まるシートは読まれない（このシート）。</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。tfl_plan(data; spec = tfl_read_table_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
+          <t>ここまでの 4 シートで table data.frame、以下の 4 シート（layout / columns / style / col_header）で列ヘッダー付きの rtftable のページまで。tfl_table_plan(data; tfl_read_table_spec(path; output_id = )) で読む。後に書いた plan_*() が勝つ。</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>tfl_plan_paginate_rows() の max_rows / split / by / min_group_rows / cont_label。先頭・末尾の空白を残すときは引用符で囲む。</t>
+          <t>plan_paginate_rows() の max_rows / split / by / min_group_rows / cont_label。先頭・末尾の空白を残すときは引用符で囲む。</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>tfl_plan_row_group() の col / mode / collapse。collapse は TRUE か列（名前・位置）の | 区切り。</t>
+          <t>plan_row_group() の col / mode / collapse。collapse は TRUE か列（名前・位置）の | 区切り。</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>group_page = TRUE で group_col の値ごとに改ページ（tfl_plan_paginate_group）。group_show = FALSE でその列を表示しない。</t>
+          <t>group_page = TRUE で group_col の値ごとに改ページ（plan_paginate_group）。group_show = FALSE でその列を表示しない。</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>tfl_plan_blanks() の where / first / last / counted。</t>
+          <t>plan_blanks() の where / first / last / counted。</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>tfl_plan_stub() の vars / into / indent / group_summary / before。</t>
+          <t>plan_stub() の vars / into / indent / group_summary / before。</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>tfl_plan_paginate_cols() の every / at / carry / order（列方向のページ分割）。</t>
+          <t>plan_paginate_cols() の every / at / carry / order（列方向のページ分割）。</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>data &lt;- tfl_ard_normalize(ard, hierarchy = c("AEBODSYS", "AEDECOD"),
+          <t>data &lt;- normalize_ard(ard, hierarchy = c("AEBODSYS", "AEDECOD"),
                       overall = "Any TEAE")</t>
         </is>
       </c>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>data &lt;- tfl_ard_normalize(ard)
+          <t>data &lt;- normalize_ard(ard)
 # row labels: the median, and the event-free probability by day (day 0 left out)
 is_time &lt;- data$variable == "time"
 data$.label[data$variable == "prob"] &lt;- "Median (95% CI)"

</xml_diff>

<commit_message>
Follow the redesigned plan verbs (rtfreporter#498, tflspec#44)
- sheets saved with the former layout columns (stub_into, group_show,
  colpages_carry, pages_by) are rewritten as they are read -- the app's
  state, study workbooks, the company standards' defaults and choices --
  so their values are not dropped by the sheet's new shape
- the company standards' built-in layout uses stub_name / group_keep
- the table builder's preview silences the notes with
  plan_cells(notes = FALSE)
- SAMPLE-01 regenerated (13 of 13 programs run); its 8 RTFs are
  byte-identical to main's
- tflplanner 0.0.1.9001: rtfreporter (>= 0.8.1.9003), tflspec (>= 0.0.23.9001)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -590,7 +590,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>cells（テンプレートでセルを作る）/ rows（統計量ごとに 1 行、生の値）。</t>
+          <t>cells（テンプレートでセルを作る）/ rows（統計量ごとに 1 行、生の値）。plan_cells(stats = )。</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>stats = rows のときの値。stat（数値）/ stat_fmt（cards 整形済み文字列）。</t>
+          <t>stats = rows のときの値。stat（数値）/ stat_fmt（cards 整形済み文字列）。plan_cells(value = )。</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>cols が複数のとき列名をつなぐ文字。既定は ____。</t>
+          <t>cols が複数のとき値の列名をつなぐ文字。既定は ____。columns シートはこの名前で列を指す。plan_columns(sep = )。</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>列方向に合計して .sort_stat 列にする統計量名。</t>
+          <t>列方向に合計して並べ替えに使う統計量名。plan_sort(stat = )。</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ページ（検査項目など）で分けた表のヘッダー {n} がどの母集団か。page = そのページの母集団（その検査を受けた人）/ table = 解析対象集団（ページキーを持たない ARD 行）。両方なら n = page | N = table で {n} と {N}。空欄 = page（両方あって食い違えば警告）。どちらも ARD に入れておくこと。</t>
+          <t>ページ（検査項目など）で分けた表のヘッダー {n} がどの母集団か。page = そのページの母集団（その検査を受けた人）/ table = 解析対象集団（ページキーを持たない ARD 行）。両方なら n = page | N = table で {n} と {N}。空欄 = page（両方あって食い違えば警告）。どちらも ARD に入れておくこと。plan_col_header(values = list(n = ...))。</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>stats = rows の帳票だけ：統計量ごとの表示桁。row = 統計量名（ラベル列の値）、digits / signif を書く（fmt_numeric と同じ）。variable / context は空欄。</t>
+          <t>stats = rows の帳票だけ：統計量ごとの表示桁。row = 統計量名（ラベル列の値）、digits / signif を書く（plan_digits(.rows = ) になる。signif は 4s のように有効桁）。variable / context は空欄。</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1056,12 +1056,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>pages_max_rows / pages_split / pages_by / pages_min_group_rows / pages_cont_label</t>
+          <t>pages_max_rows / pages_split / pages_min_group_rows / pages_cont_label</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>plan_paginate_rows() の max_rows / split / by / min_group_rows / cont_label。先頭・末尾の空白を残すときは引用符で囲む。</t>
+          <t>plan_paginate_rows() の max_rows / split / min_group_rows / cont_label。先頭・末尾の空白を残すときは引用符で囲む。値ごとの改ページは group_page。</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1078,12 +1078,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>group_col / group_mode / group_collapse</t>
+          <t>group_mode / group_collapse</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>plan_row_group() の col / mode / collapse。collapse は TRUE か列（名前・位置）の | 区切り。</t>
+          <t>plan_row_group() の mode / collapse。collapse は TRUE か列（名前・位置）の | 区切り。グループの列は行キーから決まる。</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1100,17 +1100,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>group_page / group_show</t>
+          <t>group_page / group_col / group_keep</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>group_page = TRUE で group_col の値ごとに改ページ（plan_paginate_group）。group_show = FALSE でその列を表示しない。</t>
+          <t>group_page = TRUE で group_col（空欄なら一番外の行キー）の値ごとに改ページ（plan_paginate_group の col / keep）。group_keep = FALSE でその列を表示しない。</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>TRUE / FALSE</t>
+          <t>TRUE / PARAM / FALSE</t>
         </is>
       </c>
     </row>
@@ -1144,12 +1144,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>stub_vars / stub_into / stub_indent / stub_summary / stub_before</t>
+          <t>stub_vars / stub_name / stub_indent / stub_summary / stub_before</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>plan_stub() の vars / into / indent / group_summary / before。</t>
+          <t>plan_stub() の vars / name / indent / group_summary / before。</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1 行 = 印字される列 1 つ。列は名前で指定（畳んだスタブは stub_into の名前）。.values = 展開された値の列すべて。</t>
+          <t>1 行 = 印字される列 1 つ。列は名前で指定（畳んだスタブは stub_name の名前、値の列は tables の sep でつないだ名前）。.values = 展開された値の列すべて。</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TRUE で行見出しの列。</t>
+          <t>TRUE で行見出しの列。plan_columns(row_title = )。</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1 行 = 1 帳票。border / align_count_pct / auto_width / row_height_twips / header_row_height_twips / blank_row_height_twips / font / font_size_half_points / table_align / cell_valign（rtftable と同じ引数）。</t>
+          <t>1 行 = 1 帳票。border / align_count_pct / row_height_twips / header_row_height_twips / blank_row_height_twips / font / font_size_half_points / table_align / cell_valign（plan_style と同じ引数）。auto_width は plan_columns(auto_width = ) になる。</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3198,7 +3198,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -3219,105 +3219,100 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>pages_by</t>
+          <t>pages_min_group_rows</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>pages_min_group_rows</t>
+          <t>pages_cont_label</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>pages_cont_label</t>
+          <t>group_col</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>group_col</t>
+          <t>group_mode</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>group_mode</t>
+          <t>group_collapse</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>group_collapse</t>
+          <t>group_page</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>group_page</t>
+          <t>group_keep</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>group_show</t>
+          <t>blank_where</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>blank_where</t>
+          <t>blank_first</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>blank_first</t>
+          <t>blank_last</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>blank_last</t>
+          <t>blank_counted</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>blank_counted</t>
+          <t>stub_vars</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>stub_vars</t>
+          <t>stub_name</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>stub_into</t>
+          <t>stub_indent</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>stub_indent</t>
+          <t>stub_summary</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>stub_summary</t>
+          <t>stub_before</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>stub_before</t>
+          <t>colpages_every</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>colpages_every</t>
+          <t>colpages_at</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>colpages_at</t>
+          <t>colpages_keep</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>colpages_carry</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>colpages_order</t>
         </is>
@@ -3372,7 +3367,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:U1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -3403,32 +3398,82 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>row_height_exact</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>header_row_height_twips</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>blank_row_height_twips</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>cell_padding_left_twips</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>cell_padding_right_twips</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>font</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>font_size_half_points</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>table_align</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>cell_valign</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>markup</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>blank_row_normalize</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>border_header</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>border_spanning</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>border_body</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>border_first_row</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>border_last_row</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sample study: a figure made with the designer (F-14-2-3); register_study() reads designed figures (#114)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -82,7 +82,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">table / listing / figure; blank: table.
+          <t xml:space="preserve">table / listing / figure / user (the report's own code leaves `content`: a data frame, rtftable pages, rtfplot figures or a list of them); blank: table.
 Example: listing</t>
         </r>
       </text>
@@ -825,7 +825,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -926,6 +926,12 @@
     <t xml:space="preserve">F-14-2-2</t>
   </si>
   <si>
+    <t xml:space="preserve">F-14-2-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">figure</t>
+  </si>
+  <si>
     <t xml:space="preserve">paper_size</t>
   </si>
   <si>
@@ -1085,6 +1091,12 @@
     <t xml:space="preserve">Kaplan-Meier Plot of Time to First Dermatologic Event</t>
   </si>
   <si>
+    <t xml:space="preserve">Figure 14.2.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaplan-Meier Curves of Time to First Dermatologic Event</t>
+  </si>
+  <si>
     <t xml:space="preserve">99</t>
   </si>
   <si>
@@ -1113,6 +1125,9 @@
   </si>
   <si>
     <t xml:space="preserve">x = censored.  The number at risk is that of Table 14.2.2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x = censored.  Dashed line: the median (probability 0.5).</t>
   </si>
   <si>
     <t xml:space="preserve">98</t>
@@ -1237,6 +1252,9 @@
   plot_layout(heights = c(1, tfl_num("risk_height", "km")))
 tfl_check(plot)
 content &lt;- plot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KM curves of the time to first dermatologic event (designed)</t>
   </si>
 </sst>
 </file>
@@ -1757,6 +1775,30 @@
       <c r="Q5"/>
       <c r="R5"/>
     </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6"/>
+      <c r="D6"/>
+      <c r="E6"/>
+      <c r="F6"/>
+      <c r="G6"/>
+      <c r="H6"/>
+      <c r="I6"/>
+      <c r="J6"/>
+      <c r="K6"/>
+      <c r="L6"/>
+      <c r="M6"/>
+      <c r="N6"/>
+      <c r="O6"/>
+      <c r="P6"/>
+      <c r="Q6"/>
+      <c r="R6"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -1774,52 +1816,52 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2">
@@ -1828,7 +1870,7 @@
       </c>
       <c r="B2"/>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -1851,7 +1893,7 @@
       </c>
       <c r="B3"/>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -1874,7 +1916,7 @@
       </c>
       <c r="B4"/>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
@@ -1890,6 +1932,29 @@
       <c r="O4"/>
       <c r="P4"/>
       <c r="Q4"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5"/>
+      <c r="C5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5"/>
+      <c r="E5"/>
+      <c r="F5"/>
+      <c r="G5"/>
+      <c r="H5"/>
+      <c r="I5"/>
+      <c r="J5"/>
+      <c r="K5"/>
+      <c r="L5"/>
+      <c r="M5"/>
+      <c r="N5"/>
+      <c r="O5"/>
+      <c r="P5"/>
+      <c r="Q5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1908,50 +1973,50 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3">
       <c r="A3"/>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D3"/>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -1959,49 +2024,49 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
@@ -2009,49 +2074,49 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C9"/>
       <c r="D9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" t="s">
         <v>68</v>
-      </c>
-      <c r="B11" t="s">
-        <v>66</v>
       </c>
       <c r="C11"/>
       <c r="D11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C12"/>
       <c r="D12"/>
@@ -2059,49 +2124,49 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C15"/>
       <c r="D15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C16"/>
       <c r="D16"/>
@@ -2109,40 +2174,40 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B18" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E18"/>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E19"/>
     </row>
@@ -2151,7 +2216,7 @@
         <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C20"/>
       <c r="D20"/>
@@ -2162,11 +2227,11 @@
         <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C21"/>
       <c r="D21" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E21"/>
     </row>
@@ -2175,11 +2240,11 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C22"/>
       <c r="D22" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E22"/>
     </row>
@@ -2188,11 +2253,11 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C23"/>
       <c r="D23" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E23"/>
     </row>
@@ -2201,7 +2266,7 @@
         <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C24"/>
       <c r="D24"/>
@@ -2212,11 +2277,11 @@
         <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C25"/>
       <c r="D25" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E25"/>
     </row>
@@ -2225,11 +2290,11 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C26"/>
       <c r="D26" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E26"/>
     </row>
@@ -2238,20 +2303,20 @@
         <v>30</v>
       </c>
       <c r="B27" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C27"/>
       <c r="D27" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E27"/>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C28"/>
       <c r="D28"/>
@@ -2259,40 +2324,40 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B29" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C29"/>
       <c r="D29" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E29"/>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B30" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C30"/>
       <c r="D30" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E30"/>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C31"/>
       <c r="D31" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E31"/>
     </row>
@@ -2301,7 +2366,7 @@
         <v>32</v>
       </c>
       <c r="B32" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2312,11 +2377,11 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C33"/>
       <c r="D33" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E33"/>
     </row>
@@ -2325,11 +2390,11 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C34"/>
       <c r="D34" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E34"/>
     </row>
@@ -2338,13 +2403,63 @@
         <v>32</v>
       </c>
       <c r="B35" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C35"/>
       <c r="D35" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E35"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" t="s">
+        <v>63</v>
+      </c>
+      <c r="C36"/>
+      <c r="D36"/>
+      <c r="E36"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>33</v>
+      </c>
+      <c r="B37" t="s">
+        <v>64</v>
+      </c>
+      <c r="C37"/>
+      <c r="D37" t="s">
+        <v>88</v>
+      </c>
+      <c r="E37"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>33</v>
+      </c>
+      <c r="B38" t="s">
+        <v>66</v>
+      </c>
+      <c r="C38"/>
+      <c r="D38" t="s">
+        <v>89</v>
+      </c>
+      <c r="E38"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>33</v>
+      </c>
+      <c r="B39" t="s">
+        <v>68</v>
+      </c>
+      <c r="C39"/>
+      <c r="D39" t="s">
+        <v>69</v>
+      </c>
+      <c r="E39"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2363,64 +2478,64 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C5" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
@@ -2430,49 +2545,49 @@
         <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C6" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D8"/>
       <c r="E8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C9" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
@@ -2482,24 +2597,37 @@
         <v>32</v>
       </c>
       <c r="B10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
     </row>
     <row r="11">
-      <c r="A11"/>
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
       <c r="B11" t="s">
-        <v>96</v>
+        <v>56</v>
       </c>
       <c r="C11" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
+    </row>
+    <row r="12">
+      <c r="A12"/>
+      <c r="B12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C12" t="s">
+        <v>102</v>
+      </c>
+      <c r="D12"/>
+      <c r="E12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2518,16 +2646,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -2547,16 +2675,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -2581,10 +2709,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2603,75 +2731,75 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D1" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B5" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B7" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8">
@@ -2679,7 +2807,7 @@
         <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
@@ -2689,10 +2817,10 @@
         <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="C9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D9"/>
     </row>
@@ -2701,12 +2829,22 @@
         <v>32</v>
       </c>
       <c r="B10" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="C10" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D10"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11"/>
+      <c r="D11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Sample: T-14-1-1's analyses as one ard_stack (T-14-1-1S) (#156)
T-14-1-1S has T-14-1-1's table definition and one cards::ard_stack()
analysis (STACK, .total_n = TRUE) with CONT and CAT inside it; the
column N and the total N come from the stack.  Its RTF is T-14-1-1's
but its number; the other reports are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -13,8 +13,9 @@
     <sheet name="footer" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="titles" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="footnotes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="about" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="_tflplanner" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="tokens" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="about" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="_tflplanner" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -108,8 +109,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">The program's name, joined to program_dir for {PROGRAM}; blank: {output_id}.
-Example: {output_id}</t>
+          <t xml:space="preserve">The program's name, joined to program_dir for {PROGRAM}; blank: the file name of the program that runs, {output_id} only when none is found.
+Example: t_14_1_1.R</t>
         </r>
       </text>
     </comment>
@@ -824,8 +825,57 @@
 </comments>
 </file>
 
+<file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tflspec</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The report a row belongs to. Blank: a study-wide default; a row naming a report replaces the default row with the same key (ARD analyses: the report the analysis serves).
+Example: T-14-1-1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The token's name: upper case, a letter then letters, digits or _; not one of rtfreporter's own ({PAGE}, {PROGRAM}, {DATETIME} ...).
+Example: STUDY</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">What it becomes; (none) takes a default out for this report.
+Example: ABC-123</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -1037,6 +1087,12 @@
     <t xml:space="preserve">&lt;Safety Analysis Set&gt;</t>
   </si>
   <si>
+    <t xml:space="preserve">T-14-1-1S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table 14.1.1S</t>
+  </si>
+  <si>
     <t xml:space="preserve">T-14-1-2</t>
   </si>
   <si>
@@ -1136,6 +1192,9 @@
     <t xml:space="preserve">Source: CDISC pilot study ADaM data of the pharmaverseadam R package.</t>
   </si>
   <si>
+    <t xml:space="preserve">name</t>
+  </si>
+  <si>
     <t xml:space="preserve">spec_version</t>
   </si>
   <si>
@@ -1152,6 +1211,9 @@
   </si>
   <si>
     <t xml:space="preserve">Demographic characteristics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographic characteristics (its ARD one ard_stack call)</t>
   </si>
   <si>
     <t xml:space="preserve">Subject disposition</t>
@@ -1614,6 +1676,147 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2"/>
+      <c r="B2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C2"/>
+      <c r="D2"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3"/>
+      <c r="D3"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C4"/>
+      <c r="D4"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5"/>
+      <c r="D5"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6"/>
+      <c r="D6"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7"/>
+      <c r="D7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C8"/>
+      <c r="D8" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9"/>
+      <c r="D9"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s">
+        <v>120</v>
+      </c>
+      <c r="C10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D10"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" t="s">
+        <v>123</v>
+      </c>
+      <c r="D11"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" t="s">
+        <v>124</v>
+      </c>
+      <c r="C12"/>
+      <c r="D12"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
@@ -2094,7 +2297,7 @@
       </c>
       <c r="C10"/>
       <c r="D10" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E10"/>
     </row>
@@ -2113,7 +2316,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B12" t="s">
         <v>63</v>
@@ -2124,33 +2327,33 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
         <v>64</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B14" t="s">
         <v>66</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B15" t="s">
         <v>68</v>
@@ -2163,7 +2366,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B16" t="s">
         <v>63</v>
@@ -2174,33 +2377,33 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B17" t="s">
         <v>64</v>
       </c>
       <c r="C17"/>
       <c r="D17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B18" t="s">
         <v>66</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E18"/>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B19" t="s">
         <v>68</v>
@@ -2213,7 +2416,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="B20" t="s">
         <v>63</v>
@@ -2224,7 +2427,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="B21" t="s">
         <v>64</v>
@@ -2237,7 +2440,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="B22" t="s">
         <v>66</v>
@@ -2250,7 +2453,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="B23" t="s">
         <v>68</v>
@@ -2263,7 +2466,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B24" t="s">
         <v>63</v>
@@ -2274,7 +2477,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B25" t="s">
         <v>64</v>
@@ -2287,7 +2490,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B26" t="s">
         <v>66</v>
@@ -2300,7 +2503,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B27" t="s">
         <v>68</v>
@@ -2313,7 +2516,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="B28" t="s">
         <v>63</v>
@@ -2324,33 +2527,33 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="B29" t="s">
         <v>64</v>
       </c>
       <c r="C29"/>
       <c r="D29" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E29"/>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="B30" t="s">
         <v>66</v>
       </c>
       <c r="C30"/>
       <c r="D30" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E30"/>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="B31" t="s">
         <v>68</v>
@@ -2363,7 +2566,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="B32" t="s">
         <v>63</v>
@@ -2374,7 +2577,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="B33" t="s">
         <v>64</v>
@@ -2387,7 +2590,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="B34" t="s">
         <v>66</v>
@@ -2400,7 +2603,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="B35" t="s">
         <v>68</v>
@@ -2413,7 +2616,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B36" t="s">
         <v>63</v>
@@ -2424,7 +2627,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B37" t="s">
         <v>64</v>
@@ -2437,7 +2640,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B38" t="s">
         <v>66</v>
@@ -2450,7 +2653,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B39" t="s">
         <v>68</v>
@@ -2460,6 +2663,56 @@
         <v>69</v>
       </c>
       <c r="E39"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>33</v>
+      </c>
+      <c r="B40" t="s">
+        <v>63</v>
+      </c>
+      <c r="C40"/>
+      <c r="D40"/>
+      <c r="E40"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>33</v>
+      </c>
+      <c r="B41" t="s">
+        <v>64</v>
+      </c>
+      <c r="C41"/>
+      <c r="D41" t="s">
+        <v>90</v>
+      </c>
+      <c r="E41"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>33</v>
+      </c>
+      <c r="B42" t="s">
+        <v>66</v>
+      </c>
+      <c r="C42"/>
+      <c r="D42" t="s">
+        <v>91</v>
+      </c>
+      <c r="E42"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>33</v>
+      </c>
+      <c r="B43" t="s">
+        <v>68</v>
+      </c>
+      <c r="C43"/>
+      <c r="D43" t="s">
+        <v>69</v>
+      </c>
+      <c r="E43"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2493,10 +2746,10 @@
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -2509,125 +2762,138 @@
         <v>56</v>
       </c>
       <c r="C3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
         <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B5" t="s">
         <v>56</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
         <v>56</v>
       </c>
       <c r="C6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D8"/>
       <c r="E8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B11" t="s">
         <v>56</v>
       </c>
       <c r="C11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
     </row>
     <row r="12">
-      <c r="A12"/>
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
       <c r="B12" t="s">
-        <v>101</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
         <v>102</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
+    </row>
+    <row r="13">
+      <c r="A13"/>
+      <c r="B13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C13" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13"/>
+      <c r="E13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2701,23 +2967,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B2" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
 </worksheet>
 </file>
 
@@ -2728,123 +2990,19 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2"/>
       <c r="B2" t="s">
-        <v>107</v>
-      </c>
-      <c r="C2"/>
-      <c r="D2"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B3" t="s">
-        <v>108</v>
-      </c>
-      <c r="C3"/>
-      <c r="D3"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B4" t="s">
-        <v>109</v>
-      </c>
-      <c r="C4"/>
-      <c r="D4"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C5"/>
-      <c r="D5"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C6"/>
-      <c r="D6" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>83</v>
-      </c>
-      <c r="B7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C7"/>
-      <c r="D7" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" t="s">
-        <v>115</v>
-      </c>
-      <c r="C8"/>
-      <c r="D8"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" t="s">
-        <v>116</v>
-      </c>
-      <c r="C9" t="s">
-        <v>117</v>
-      </c>
-      <c r="D9"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" t="s">
-        <v>118</v>
-      </c>
-      <c r="C10" t="s">
-        <v>119</v>
-      </c>
-      <c r="D10"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" t="s">
-        <v>120</v>
-      </c>
-      <c r="C11"/>
-      <c r="D11"/>
+        <v>56</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
2-1 lists the report's own analysis data; the sample's tables read analysis data
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -875,7 +875,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="128">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -1207,10 +1207,19 @@
     <t xml:space="preserve">process_code</t>
   </si>
   <si>
+    <t xml:space="preserve">section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">population</t>
+  </si>
+  <si>
     <t xml:space="preserve">(every report)</t>
   </si>
   <si>
     <t xml:space="preserve">Demographic characteristics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAF</t>
   </si>
   <si>
     <t xml:space="preserve">Demographic characteristics (its ARD one ard_stack call)</t>
@@ -1694,65 +1703,93 @@
       <c r="D1" t="s">
         <v>109</v>
       </c>
+      <c r="E1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F1" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
         <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
+      <c r="E3"/>
+      <c r="F3" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
         <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
+      <c r="E4"/>
+      <c r="F4" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
         <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
+      <c r="E5"/>
+      <c r="F5" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
         <v>75</v>
       </c>
       <c r="B6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
+      <c r="E6"/>
+      <c r="F6" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
         <v>78</v>
       </c>
       <c r="B7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>116</v>
+        <v>119</v>
+      </c>
+      <c r="E7"/>
+      <c r="F7" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="8">
@@ -1760,11 +1797,15 @@
         <v>85</v>
       </c>
       <c r="B8" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>118</v>
+        <v>121</v>
+      </c>
+      <c r="E8"/>
+      <c r="F8" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="9">
@@ -1772,44 +1813,52 @@
         <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
+      <c r="E9"/>
+      <c r="F9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
         <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C10" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
         <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C11" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C12"/>
       <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
An analysis data is a report's: 2-1, copy from another report, the Data tab without them, the sample by report; 0.0.2.9108
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -875,7 +875,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -1211,6 +1211,9 @@
   </si>
   <si>
     <t xml:space="preserve">population</t>
+  </si>
+  <si>
+    <t xml:space="preserve">datasets</t>
   </si>
   <si>
     <t xml:space="preserve">(every report)</t>
@@ -1709,156 +1712,170 @@
       <c r="F1" t="s">
         <v>111</v>
       </c>
+      <c r="G1" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
       <c r="E2"/>
       <c r="F2"/>
+      <c r="G2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
         <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
       <c r="E3"/>
       <c r="F3" t="s">
-        <v>114</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="G3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
         <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>114</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="G4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
         <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>114</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="G5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
         <v>75</v>
       </c>
       <c r="B6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>114</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="G6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
         <v>78</v>
       </c>
       <c r="B7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>114</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="G7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
         <v>85</v>
       </c>
       <c r="B8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>114</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="G8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
         <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
       <c r="E9"/>
       <c r="F9"/>
+      <c r="G9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
         <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
       <c r="F10"/>
+      <c r="G10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
         <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
       <c r="F11"/>
+      <c r="G11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C12"/>
       <c r="D12"/>
       <c r="E12"/>
       <c r="F12"/>
+      <c r="G12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
The report programs, tidied: their head, the data part, the study's header, a figure's plot (#275)
- Head: the banner and one stopifnot(); the report's id is report_id.
- Data part: one heading; the default table_data / table_process without
  the "Leaves ...", "Input data are in ..." and commented-out lines; the
  table's saveRDS() at its end.
- A figure's plot to the report as it is: rtf_figures(doc, plot)
  (rtfreporter >= 0.8.2.9029).
- save_ard(..., definition = ) and record_report() (were .save_output(),
  .record_report()); the ARD banner shorter; batch.R's lists indented.
- report_setup.R writes the study's header and footer also when the
  study has default header or footer rows; the sample's header is
  tokens, so its reports use study_header (the RTFs are the same).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -456,12 +456,25 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
+          <t xml:space="preserve">The document's font (its font table); the study's row (blank output_id) is the company's, written once in the setup code; blank: rtfreporter's option (Courier).
+Example: Courier New</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
           <t xml:space="preserve">The body font size in half-points (18 = 9 pt); blank: rtfreporter's option.
 Example: 18</t>
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -474,7 +487,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -487,7 +500,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -500,7 +513,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -513,7 +526,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -875,7 +888,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -1012,6 +1025,9 @@
     <t xml:space="preserve">footer_dist_in</t>
   </si>
   <si>
+    <t xml:space="preserve">font</t>
+  </si>
+  <si>
     <t xml:space="preserve">font_size_half_points</t>
   </si>
   <si>
@@ -1063,136 +1079,121 @@
     <t xml:space="preserve">Page {PAGE} of {TOTAL_PAGES}</t>
   </si>
   <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{OUTPUT_LABEL}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{OUTPUT_TITLE}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;{OUTPUT_POPULATION}&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{PROGRAM}       Generated on: {DATETIME}</t>
+  </si>
+  <si>
     <t xml:space="preserve">T-14-1-1</t>
   </si>
   <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table 14.1.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
+    <t xml:space="preserve">SD = Standard Deviation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-1-1S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-2-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SD = Standard Deviation; SE = Standard Error; CI = Confidence Interval (t distribution).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-3-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subjects are counted once per system organ class and once per preferred term.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vertical bars: mean +/- SE.  Systolic blood pressure after 5 minutes lying down.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Systolic blood pressure after 5 minutes lying down.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-2-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dermatologic event: first treatment-emergent skin and subcutaneous tissue disorder or application site event; censored at the end of treatment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaplan-Meier estimates; 95% CI of the median by the Brookmeyer-Crowley method (log transformation). NE = not estimable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x = censored.  The number at risk is that of Table 14.2.2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x = censored.  Dashed line: the median (probability 0.5).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: CDISC pilot study ADaM data of the pharmaverseadam R package.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUTPUT_TITLE</t>
   </si>
   <si>
     <t xml:space="preserve">Demographic Characteristics</t>
   </si>
   <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;Safety Analysis Set&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-1-1S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table 14.1.1S</t>
+    <t xml:space="preserve">OUTPUT_POPULATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safety Analysis Set</t>
   </si>
   <si>
     <t xml:space="preserve">T-14-1-2</t>
   </si>
   <si>
-    <t xml:space="preserve">Table 14.1.2</t>
-  </si>
-  <si>
     <t xml:space="preserve">Subject Disposition</t>
   </si>
   <si>
-    <t xml:space="preserve">T-14-2-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table 14.2.1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Systolic Blood Pressure (mmHg): Change from Baseline at Week 24</t>
   </si>
   <si>
-    <t xml:space="preserve">T-14-3-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table 14.3.1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Treatment-Emergent Adverse Events by System Organ Class and Preferred Term</t>
   </si>
   <si>
-    <t xml:space="preserve">Listing 16.2.7</t>
-  </si>
-  <si>
     <t xml:space="preserve">Severe Treatment-Emergent Adverse Events</t>
   </si>
   <si>
-    <t xml:space="preserve">Figure 14.2.1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Mean (SE) Change from Baseline in Systolic Blood Pressure over Time</t>
   </si>
   <si>
-    <t xml:space="preserve">T-14-2-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table 14.2.2</t>
-  </si>
-  <si>
     <t xml:space="preserve">Time to First Dermatologic Event: Kaplan-Meier Estimates</t>
   </si>
   <si>
-    <t xml:space="preserve">Figure 14.2.2</t>
-  </si>
-  <si>
     <t xml:space="preserve">Kaplan-Meier Plot of Time to First Dermatologic Event</t>
   </si>
   <si>
-    <t xml:space="preserve">Figure 14.2.3</t>
-  </si>
-  <si>
     <t xml:space="preserve">Kaplan-Meier Curves of Time to First Dermatologic Event</t>
-  </si>
-  <si>
-    <t xml:space="preserve">99</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{PROGRAM}       Generated on: {DATETIME}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SD = Standard Deviation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SD = Standard Deviation; SE = Standard Error; CI = Confidence Interval (t distribution).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subjects are counted once per system organ class and once per preferred term.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vertical bars: mean +/- SE.  Systolic blood pressure after 5 minutes lying down.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Systolic blood pressure after 5 minutes lying down.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dermatologic event: first treatment-emergent skin and subcutaneous tissue disorder or application site event; censored at the end of treatment.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kaplan-Meier estimates; 95% CI of the median by the Brookmeyer-Crowley method (log transformation). NE = not estimable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">x = censored.  The number at risk is that of Table 14.2.2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">x = censored.  Dashed line: the median (probability 0.5).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">98</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source: CDISC pilot study ADaM data of the pharmaverseadam R package.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">name</t>
   </si>
   <si>
     <t xml:space="preserve">spec_version</t>
@@ -1699,28 +1700,28 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F1" t="s">
         <v>107</v>
       </c>
-      <c r="C1" t="s">
+      <c r="G1" t="s">
         <v>108</v>
-      </c>
-      <c r="D1" t="s">
-        <v>109</v>
-      </c>
-      <c r="E1" t="s">
-        <v>110</v>
-      </c>
-      <c r="F1" t="s">
-        <v>111</v>
-      </c>
-      <c r="G1" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
@@ -1730,46 +1731,46 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="B3" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
       <c r="E3"/>
       <c r="F3" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G5"/>
     </row>
@@ -1778,47 +1779,47 @@
         <v>75</v>
       </c>
       <c r="B6" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B7" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B8" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G8"/>
     </row>
@@ -1827,7 +1828,7 @@
         <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
@@ -1840,10 +1841,10 @@
         <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C10" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
@@ -1855,10 +1856,10 @@
         <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C11" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
@@ -1870,7 +1871,7 @@
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C12"/>
       <c r="D12"/>
@@ -2133,6 +2134,9 @@
       <c r="Q1" t="s">
         <v>50</v>
       </c>
+      <c r="R1" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -2140,7 +2144,7 @@
       </c>
       <c r="B2"/>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -2156,6 +2160,7 @@
       <c r="O2"/>
       <c r="P2"/>
       <c r="Q2"/>
+      <c r="R2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -2163,7 +2168,7 @@
       </c>
       <c r="B3"/>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -2179,6 +2184,7 @@
       <c r="O3"/>
       <c r="P3"/>
       <c r="Q3"/>
+      <c r="R3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
@@ -2186,7 +2192,7 @@
       </c>
       <c r="B4"/>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
@@ -2202,6 +2208,7 @@
       <c r="O4"/>
       <c r="P4"/>
       <c r="Q4"/>
+      <c r="R4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
@@ -2209,7 +2216,7 @@
       </c>
       <c r="B5"/>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
@@ -2225,6 +2232,7 @@
       <c r="O5"/>
       <c r="P5"/>
       <c r="Q5"/>
+      <c r="R5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2243,48 +2251,46 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3"/>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D3"/>
       <c r="E3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s">
-        <v>62</v>
-      </c>
+      <c r="A4"/>
       <c r="B4" t="s">
         <v>63</v>
       </c>
@@ -2293,9 +2299,7 @@
       <c r="E4"/>
     </row>
     <row r="5">
-      <c r="A5" t="s">
-        <v>62</v>
-      </c>
+      <c r="A5"/>
       <c r="B5" t="s">
         <v>64</v>
       </c>
@@ -2306,9 +2310,7 @@
       <c r="E5"/>
     </row>
     <row r="6">
-      <c r="A6" t="s">
-        <v>62</v>
-      </c>
+      <c r="A6"/>
       <c r="B6" t="s">
         <v>66</v>
       </c>
@@ -2319,9 +2321,7 @@
       <c r="E6"/>
     </row>
     <row r="7">
-      <c r="A7" t="s">
-        <v>62</v>
-      </c>
+      <c r="A7"/>
       <c r="B7" t="s">
         <v>68</v>
       </c>
@@ -2330,456 +2330,6 @@
         <v>69</v>
       </c>
       <c r="E7"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>70</v>
-      </c>
-      <c r="B8" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8"/>
-      <c r="D8"/>
-      <c r="E8"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>70</v>
-      </c>
-      <c r="B9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C9"/>
-      <c r="D9" t="s">
-        <v>71</v>
-      </c>
-      <c r="E9"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>70</v>
-      </c>
-      <c r="B10" t="s">
-        <v>66</v>
-      </c>
-      <c r="C10"/>
-      <c r="D10" t="s">
-        <v>67</v>
-      </c>
-      <c r="E10"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>70</v>
-      </c>
-      <c r="B11" t="s">
-        <v>68</v>
-      </c>
-      <c r="C11"/>
-      <c r="D11" t="s">
-        <v>69</v>
-      </c>
-      <c r="E11"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>72</v>
-      </c>
-      <c r="B12" t="s">
-        <v>63</v>
-      </c>
-      <c r="C12"/>
-      <c r="D12"/>
-      <c r="E12"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>72</v>
-      </c>
-      <c r="B13" t="s">
-        <v>64</v>
-      </c>
-      <c r="C13"/>
-      <c r="D13" t="s">
-        <v>73</v>
-      </c>
-      <c r="E13"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>72</v>
-      </c>
-      <c r="B14" t="s">
-        <v>66</v>
-      </c>
-      <c r="C14"/>
-      <c r="D14" t="s">
-        <v>74</v>
-      </c>
-      <c r="E14"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>72</v>
-      </c>
-      <c r="B15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C15"/>
-      <c r="D15" t="s">
-        <v>69</v>
-      </c>
-      <c r="E15"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="s">
-        <v>75</v>
-      </c>
-      <c r="B16" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16"/>
-      <c r="D16"/>
-      <c r="E16"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>75</v>
-      </c>
-      <c r="B17" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17"/>
-      <c r="D17" t="s">
-        <v>76</v>
-      </c>
-      <c r="E17"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
-        <v>75</v>
-      </c>
-      <c r="B18" t="s">
-        <v>66</v>
-      </c>
-      <c r="C18"/>
-      <c r="D18" t="s">
-        <v>77</v>
-      </c>
-      <c r="E18"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="s">
-        <v>75</v>
-      </c>
-      <c r="B19" t="s">
-        <v>68</v>
-      </c>
-      <c r="C19"/>
-      <c r="D19" t="s">
-        <v>69</v>
-      </c>
-      <c r="E19"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>78</v>
-      </c>
-      <c r="B20" t="s">
-        <v>63</v>
-      </c>
-      <c r="C20"/>
-      <c r="D20"/>
-      <c r="E20"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="s">
-        <v>78</v>
-      </c>
-      <c r="B21" t="s">
-        <v>64</v>
-      </c>
-      <c r="C21"/>
-      <c r="D21" t="s">
-        <v>79</v>
-      </c>
-      <c r="E21"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>78</v>
-      </c>
-      <c r="B22" t="s">
-        <v>66</v>
-      </c>
-      <c r="C22"/>
-      <c r="D22" t="s">
-        <v>80</v>
-      </c>
-      <c r="E22"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
-        <v>78</v>
-      </c>
-      <c r="B23" t="s">
-        <v>68</v>
-      </c>
-      <c r="C23"/>
-      <c r="D23" t="s">
-        <v>69</v>
-      </c>
-      <c r="E23"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="s">
-        <v>28</v>
-      </c>
-      <c r="B24" t="s">
-        <v>63</v>
-      </c>
-      <c r="C24"/>
-      <c r="D24"/>
-      <c r="E24"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="s">
-        <v>28</v>
-      </c>
-      <c r="B25" t="s">
-        <v>64</v>
-      </c>
-      <c r="C25"/>
-      <c r="D25" t="s">
-        <v>81</v>
-      </c>
-      <c r="E25"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="s">
-        <v>28</v>
-      </c>
-      <c r="B26" t="s">
-        <v>66</v>
-      </c>
-      <c r="C26"/>
-      <c r="D26" t="s">
-        <v>82</v>
-      </c>
-      <c r="E26"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" t="s">
-        <v>68</v>
-      </c>
-      <c r="C27"/>
-      <c r="D27" t="s">
-        <v>69</v>
-      </c>
-      <c r="E27"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28"/>
-      <c r="D28"/>
-      <c r="E28"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" t="s">
-        <v>64</v>
-      </c>
-      <c r="C29"/>
-      <c r="D29" t="s">
-        <v>83</v>
-      </c>
-      <c r="E29"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" t="s">
-        <v>66</v>
-      </c>
-      <c r="C30"/>
-      <c r="D30" t="s">
-        <v>84</v>
-      </c>
-      <c r="E30"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="s">
-        <v>30</v>
-      </c>
-      <c r="B31" t="s">
-        <v>68</v>
-      </c>
-      <c r="C31"/>
-      <c r="D31" t="s">
-        <v>69</v>
-      </c>
-      <c r="E31"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="s">
-        <v>85</v>
-      </c>
-      <c r="B32" t="s">
-        <v>63</v>
-      </c>
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="s">
-        <v>85</v>
-      </c>
-      <c r="B33" t="s">
-        <v>64</v>
-      </c>
-      <c r="C33"/>
-      <c r="D33" t="s">
-        <v>86</v>
-      </c>
-      <c r="E33"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="s">
-        <v>85</v>
-      </c>
-      <c r="B34" t="s">
-        <v>66</v>
-      </c>
-      <c r="C34"/>
-      <c r="D34" t="s">
-        <v>87</v>
-      </c>
-      <c r="E34"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="s">
-        <v>85</v>
-      </c>
-      <c r="B35" t="s">
-        <v>68</v>
-      </c>
-      <c r="C35"/>
-      <c r="D35" t="s">
-        <v>69</v>
-      </c>
-      <c r="E35"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="s">
-        <v>32</v>
-      </c>
-      <c r="B36" t="s">
-        <v>63</v>
-      </c>
-      <c r="C36"/>
-      <c r="D36"/>
-      <c r="E36"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="s">
-        <v>32</v>
-      </c>
-      <c r="B37" t="s">
-        <v>64</v>
-      </c>
-      <c r="C37"/>
-      <c r="D37" t="s">
-        <v>88</v>
-      </c>
-      <c r="E37"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="s">
-        <v>32</v>
-      </c>
-      <c r="B38" t="s">
-        <v>66</v>
-      </c>
-      <c r="C38"/>
-      <c r="D38" t="s">
-        <v>89</v>
-      </c>
-      <c r="E38"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="s">
-        <v>32</v>
-      </c>
-      <c r="B39" t="s">
-        <v>68</v>
-      </c>
-      <c r="C39"/>
-      <c r="D39" t="s">
-        <v>69</v>
-      </c>
-      <c r="E39"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="s">
-        <v>33</v>
-      </c>
-      <c r="B40" t="s">
-        <v>63</v>
-      </c>
-      <c r="C40"/>
-      <c r="D40"/>
-      <c r="E40"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="s">
-        <v>33</v>
-      </c>
-      <c r="B41" t="s">
-        <v>64</v>
-      </c>
-      <c r="C41"/>
-      <c r="D41" t="s">
-        <v>90</v>
-      </c>
-      <c r="E41"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="s">
-        <v>33</v>
-      </c>
-      <c r="B42" t="s">
-        <v>66</v>
-      </c>
-      <c r="C42"/>
-      <c r="D42" t="s">
-        <v>91</v>
-      </c>
-      <c r="E42"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="s">
-        <v>33</v>
-      </c>
-      <c r="B43" t="s">
-        <v>68</v>
-      </c>
-      <c r="C43"/>
-      <c r="D43" t="s">
-        <v>69</v>
-      </c>
-      <c r="E43"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2798,51 +2348,51 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>71</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C4" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
@@ -2852,23 +2402,23 @@
         <v>75</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" t="s">
         <v>78</v>
-      </c>
-      <c r="B6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" t="s">
-        <v>96</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
@@ -2878,10 +2428,10 @@
         <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
@@ -2891,36 +2441,36 @@
         <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C8" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="D8"/>
       <c r="E8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C9" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C10" t="s">
-        <v>100</v>
+        <v>83</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
@@ -2930,10 +2480,10 @@
         <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
@@ -2943,10 +2493,10 @@
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C12" t="s">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
@@ -2954,10 +2504,10 @@
     <row r="13">
       <c r="A13"/>
       <c r="B13" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="C13" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
@@ -2979,16 +2529,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -3008,16 +2558,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -3037,10 +2587,230 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" t="s">
+        <v>91</v>
+      </c>
+      <c r="C13" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" t="s">
+        <v>89</v>
+      </c>
+      <c r="C20" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -3065,10 +2835,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Four more sample reports: the ARD's rows a table does not use, CI with text statistics, no analysis set, an analysis set by a condition
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -888,7 +888,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="143">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -1121,6 +1121,27 @@
     <t xml:space="preserve">SD = Standard Deviation; SE = Standard Error; CI = Confidence Interval (t distribution).</t>
   </si>
   <si>
+    <t xml:space="preserve">T-14-0-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The dictionary versions are the study's (data management plan); the dates are those of ADSL.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-1-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SD = Standard Deviation.  Screen failures: subjects not randomized (ARM is Screen Failure).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-2-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI = Confidence Interval.  95% CI and p-value: one-sample t-test of the change from baseline (H0: mean change = 0).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Systolic blood pressure after 5 minutes lying down.</t>
+  </si>
+  <si>
     <t xml:space="preserve">T-14-3-1</t>
   </si>
   <si>
@@ -1130,9 +1151,6 @@
     <t xml:space="preserve">Vertical bars: mean +/- SE.  Systolic blood pressure after 5 minutes lying down.</t>
   </si>
   <si>
-    <t xml:space="preserve">Systolic blood pressure after 5 minutes lying down.</t>
-  </si>
-  <si>
     <t xml:space="preserve">T-14-2-2</t>
   </si>
   <si>
@@ -1178,6 +1196,27 @@
     <t xml:space="preserve">Systolic Blood Pressure (mmHg): Change from Baseline at Week 24</t>
   </si>
   <si>
+    <t xml:space="preserve">T-14-1-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age Group and Sex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Study Information</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Subjects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographic Characteristics of Screen Failures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Screen Failures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Systolic Blood Pressure (mmHg): Mean Change from Baseline at Week 24 (95% CI)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Treatment-Emergent Adverse Events by System Organ Class and Preferred Term</t>
   </si>
   <si>
@@ -1220,6 +1259,15 @@
     <t xml:space="preserve">(every report)</t>
   </si>
   <si>
+    <t xml:space="preserve">Study information: dictionary versions and the dates of the data (no analysis set)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographic characteristics of the screen failures (an analysis set by a condition alone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCRF</t>
+  </si>
+  <si>
     <t xml:space="preserve">Demographic characteristics</t>
   </si>
   <si>
@@ -1233,6 +1281,12 @@
   </si>
   <si>
     <t xml:space="preserve">Systolic blood pressure: change from baseline at Week 24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age group and sex: the ARD keeps cards' default n, N and p; the table prints n (%) and leaves the N rows out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Systolic blood pressure: mean change at Week 24 (95% CI), p-value; the ARD also holds the test's method and alternative as text</t>
   </si>
   <si>
     <t xml:space="preserve">TEAEs by SOC / PT</t>
@@ -1700,28 +1754,28 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="C1" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="D1" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="E1" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="F1" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="G1" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
@@ -1731,153 +1785,211 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B3" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
       <c r="E3"/>
-      <c r="F3" t="s">
-        <v>111</v>
-      </c>
+      <c r="F3"/>
       <c r="G3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B4" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="G4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="G5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="G6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="B7" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="C7"/>
-      <c r="D7" t="s">
-        <v>116</v>
-      </c>
+      <c r="D7"/>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="G7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C8"/>
-      <c r="D8" t="s">
-        <v>118</v>
-      </c>
+      <c r="D8"/>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="G8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>102</v>
       </c>
       <c r="B9" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
       <c r="E9"/>
-      <c r="F9"/>
+      <c r="F9" t="s">
+        <v>127</v>
+      </c>
       <c r="G9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
-      </c>
-      <c r="C10" t="s">
-        <v>121</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="C10"/>
       <c r="D10"/>
       <c r="E10"/>
-      <c r="F10"/>
+      <c r="F10" t="s">
+        <v>127</v>
+      </c>
       <c r="G10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>84</v>
       </c>
       <c r="B11" t="s">
-        <v>122</v>
-      </c>
-      <c r="C11" t="s">
-        <v>123</v>
-      </c>
-      <c r="D11"/>
+        <v>133</v>
+      </c>
+      <c r="C11"/>
+      <c r="D11" t="s">
+        <v>134</v>
+      </c>
       <c r="E11"/>
-      <c r="F11"/>
+      <c r="F11" t="s">
+        <v>127</v>
+      </c>
       <c r="G11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>87</v>
+      </c>
+      <c r="B12" t="s">
+        <v>135</v>
+      </c>
+      <c r="C12"/>
+      <c r="D12" t="s">
+        <v>136</v>
+      </c>
+      <c r="E12"/>
+      <c r="F12" t="s">
+        <v>127</v>
+      </c>
+      <c r="G12"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" t="s">
+        <v>137</v>
+      </c>
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13"/>
+      <c r="F13"/>
+      <c r="G13"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" t="s">
+        <v>138</v>
+      </c>
+      <c r="C14" t="s">
+        <v>139</v>
+      </c>
+      <c r="D14"/>
+      <c r="E14"/>
+      <c r="F14"/>
+      <c r="G14"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" t="s">
+        <v>140</v>
+      </c>
+      <c r="C15" t="s">
+        <v>141</v>
+      </c>
+      <c r="D15"/>
+      <c r="E15"/>
+      <c r="F15"/>
+      <c r="G15"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
         <v>33</v>
       </c>
-      <c r="B12" t="s">
-        <v>124</v>
-      </c>
-      <c r="C12"/>
-      <c r="D12"/>
-      <c r="E12"/>
-      <c r="F12"/>
-      <c r="G12"/>
+      <c r="B16" t="s">
+        <v>142</v>
+      </c>
+      <c r="C16"/>
+      <c r="D16"/>
+      <c r="E16"/>
+      <c r="F16"/>
+      <c r="G16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2425,26 +2537,26 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="B7" t="s">
         <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B8" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D8"/>
       <c r="E8"/>
@@ -2454,63 +2566,115 @@
         <v>81</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B10" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
         <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
     </row>
     <row r="13">
-      <c r="A13"/>
+      <c r="A13" t="s">
+        <v>87</v>
+      </c>
       <c r="B13" t="s">
-        <v>86</v>
+        <v>57</v>
       </c>
       <c r="C13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14"/>
+      <c r="E14"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" t="s">
+        <v>90</v>
+      </c>
+      <c r="D15"/>
+      <c r="E15"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" t="s">
+        <v>91</v>
+      </c>
+      <c r="D16"/>
+      <c r="E16"/>
+    </row>
+    <row r="17">
+      <c r="A17"/>
+      <c r="B17" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17"/>
+      <c r="E17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2587,7 +2751,7 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -2598,10 +2762,10 @@
         <v>72</v>
       </c>
       <c r="B2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3">
@@ -2609,10 +2773,10 @@
         <v>72</v>
       </c>
       <c r="B3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4">
@@ -2620,10 +2784,10 @@
         <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5">
@@ -2631,32 +2795,32 @@
         <v>74</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B6" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C6" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B7" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8">
@@ -2664,10 +2828,10 @@
         <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9">
@@ -2675,76 +2839,76 @@
         <v>75</v>
       </c>
       <c r="B9" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C9" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="B10" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C10" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="B11" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C11" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="B12" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C12" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C13" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="B14" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C14" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="B15" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16">
@@ -2752,10 +2916,10 @@
         <v>81</v>
       </c>
       <c r="B16" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C16" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17">
@@ -2763,54 +2927,142 @@
         <v>81</v>
       </c>
       <c r="B17" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C17" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>32</v>
+        <v>84</v>
       </c>
       <c r="B18" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C18" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>84</v>
       </c>
       <c r="B19" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C19" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="C20" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" t="s">
+        <v>97</v>
+      </c>
+      <c r="C21" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C23" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>87</v>
+      </c>
+      <c r="B24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C24" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>87</v>
+      </c>
+      <c r="B25" t="s">
+        <v>97</v>
+      </c>
+      <c r="C25" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" t="s">
+        <v>95</v>
+      </c>
+      <c r="C26" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
         <v>33</v>
       </c>
-      <c r="B21" t="s">
-        <v>91</v>
-      </c>
-      <c r="C21" t="s">
-        <v>92</v>
+      <c r="B28" t="s">
+        <v>95</v>
+      </c>
+      <c r="C28" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" t="s">
+        <v>97</v>
+      </c>
+      <c r="C29" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -2835,7 +3087,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="B2" t="s">
         <v>57</v>

</xml_diff>

<commit_message>
A figure prints a table's numbers: its ARD source, the ARD pieces (#293)
A figure's step 2 chooses its ARD: none, its own analyses, or a table's
(report row ard_source = table:<id>; set_fig_ard_source()), with the
table's analyses and statistics shown.  The program reads it as ard at
the top of '# ---- data ----'; the Plot Designer offers the ARD pieces
(ard_number, ard_stats) when the figure has one, with the ARD's analyses,
variables and statistics as choices; the preview draws them.  The spec
check names a source that is not a table, a design reading an ARD
without one, an ARD not made yet (warning) and pieces the ARD cannot
answer.  rename_output() of a table renames its figures' references.
The sample's F-14-2-3 prints T-14-2-2's medians.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -278,7 +278,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Where the report's ARD comes from: blank, its own ARD definition (the analyses rows of its output_id); import:&lt;file&gt;, an ARD made elsewhere and taken in (the file in the study's input/ard/ folder, read with tfl_read_ard()).
+          <t xml:space="preserve">Where the report's ARD comes from: blank (a figure: none), its own ARD definition (the analyses rows of its output_id; a figure: own); import:&lt;file&gt;, an ARD made elsewhere and taken in (the file in the study's input/ard/ folder, read with tfl_read_ard()); table:&lt;output_id&gt;, a figure's: that table's ARD.
 Example: import:t_14_2_1_cro.json</t>
         </r>
       </text>
@@ -888,7 +888,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="145">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -995,6 +995,9 @@
     <t xml:space="preserve">figure</t>
   </si>
   <si>
+    <t xml:space="preserve">table:T-14-2-2</t>
+  </si>
+  <si>
     <t xml:space="preserve">paper_size</t>
   </si>
   <si>
@@ -1163,7 +1166,7 @@
     <t xml:space="preserve">x = censored.  The number at risk is that of Table 14.2.2.</t>
   </si>
   <si>
-    <t xml:space="preserve">x = censored.  Dashed line: the median (probability 0.5).</t>
+    <t xml:space="preserve">x = censored.  Dashed line: the median (probability 0.5).  The medians are those of Table 14.2.2.</t>
   </si>
   <si>
     <t xml:space="preserve">98</t>
@@ -1254,6 +1257,9 @@
   </si>
   <si>
     <t xml:space="preserve">datasets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">batches</t>
   </si>
   <si>
     <t xml:space="preserve">(every report)</t>
@@ -1754,242 +1760,260 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G1" t="s">
-        <v>121</v>
+        <v>122</v>
+      </c>
+      <c r="H1" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
       <c r="E2"/>
       <c r="F2"/>
       <c r="G2"/>
+      <c r="H2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
       <c r="E3"/>
       <c r="F3"/>
       <c r="G3"/>
+      <c r="H3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B4" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G4"/>
+      <c r="H4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G5"/>
+      <c r="H5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G6"/>
+      <c r="H6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C7"/>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G7"/>
+      <c r="H7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G8"/>
+      <c r="H8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B9" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G9"/>
+      <c r="H9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C10"/>
       <c r="D10"/>
       <c r="E10"/>
       <c r="F10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G10"/>
+      <c r="H10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C11"/>
       <c r="D11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E11"/>
       <c r="F11" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G11"/>
+      <c r="H11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C12"/>
       <c r="D12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E12"/>
       <c r="F12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G12"/>
+      <c r="H12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
         <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C13"/>
       <c r="D13"/>
       <c r="E13"/>
       <c r="F13"/>
       <c r="G13"/>
+      <c r="H13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
         <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C14" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D14"/>
       <c r="E14"/>
       <c r="F14"/>
       <c r="G14"/>
+      <c r="H14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
         <v>32</v>
       </c>
       <c r="B15" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C15" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D15"/>
       <c r="E15"/>
       <c r="F15"/>
       <c r="G15"/>
+      <c r="H15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
         <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C16"/>
       <c r="D16"/>
       <c r="E16"/>
       <c r="F16"/>
       <c r="G16"/>
+      <c r="H16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2179,7 +2203,9 @@
       <c r="N6"/>
       <c r="O6"/>
       <c r="P6"/>
-      <c r="Q6"/>
+      <c r="Q6" t="s">
+        <v>35</v>
+      </c>
       <c r="R6"/>
     </row>
   </sheetData>
@@ -2199,55 +2225,55 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
@@ -2256,7 +2282,7 @@
       </c>
       <c r="B2"/>
       <c r="C2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -2280,7 +2306,7 @@
       </c>
       <c r="B3"/>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -2304,7 +2330,7 @@
       </c>
       <c r="B4"/>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
@@ -2328,7 +2354,7 @@
       </c>
       <c r="B5"/>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
@@ -2363,48 +2389,48 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
       <c r="A3"/>
       <c r="B3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D3"/>
       <c r="E3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4">
       <c r="A4"/>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -2413,33 +2439,33 @@
     <row r="5">
       <c r="A5"/>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6"/>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7"/>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E7"/>
     </row>
@@ -2460,129 +2486,129 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" t="s">
         <v>74</v>
-      </c>
-      <c r="B4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C4" t="s">
-        <v>73</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D8"/>
       <c r="E8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
@@ -2592,49 +2618,49 @@
         <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D14"/>
       <c r="E14"/>
@@ -2644,10 +2670,10 @@
         <v>32</v>
       </c>
       <c r="B15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D15"/>
       <c r="E15"/>
@@ -2657,10 +2683,10 @@
         <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D16"/>
       <c r="E16"/>
@@ -2668,10 +2694,10 @@
     <row r="17">
       <c r="A17"/>
       <c r="B17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C17" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D17"/>
       <c r="E17"/>
@@ -2693,16 +2719,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -2722,16 +2748,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -2751,7 +2777,7 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -2759,200 +2785,200 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C7" t="s">
         <v>99</v>
-      </c>
-      <c r="B7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C7" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C11" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B15" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B16" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B17" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C17" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C19" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20">
@@ -2960,10 +2986,10 @@
         <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21">
@@ -2971,10 +2997,10 @@
         <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C21" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22">
@@ -2982,10 +3008,10 @@
         <v>30</v>
       </c>
       <c r="B22" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C22" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23">
@@ -2993,32 +3019,32 @@
         <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C23" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B24" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C24" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B25" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C25" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26">
@@ -3026,10 +3052,10 @@
         <v>32</v>
       </c>
       <c r="B26" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C26" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="27">
@@ -3037,10 +3063,10 @@
         <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C27" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="28">
@@ -3048,10 +3074,10 @@
         <v>33</v>
       </c>
       <c r="B28" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C28" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="29">
@@ -3059,10 +3085,10 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -3087,10 +3113,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Race with its Asian sub-categories, nested (T-14-1-5) or in two blocks (T-14-1-6); the builder's 'under' field
The builder's variable form: a categorical variable's rows under a level
of another (variables$under, plan_nest()).  The sample: an Enrolled
analysis set (ENR), analysis data with a demonstration sub-race of Asian
and a Total column, the two tables from the same analyses; the other
tables are byte-identical.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -888,7 +888,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="155">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -1136,6 +1136,18 @@
     <t xml:space="preserve">SD = Standard Deviation.  Screen failures: subjects not randomized (ARM is Screen Failure).</t>
   </si>
   <si>
+    <t xml:space="preserve">T-14-1-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enrolled subjects: all subjects of ADSL, screen failures included.  Percentages of the column's subjects.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asian sub-categories (Chinese, Japanese, Korean) are derived for demonstration; they are not in the source data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-1-6</t>
+  </si>
+  <si>
     <t xml:space="preserve">T-14-2-3</t>
   </si>
   <si>
@@ -1217,6 +1229,15 @@
     <t xml:space="preserve">All Screen Failures</t>
   </si>
   <si>
+    <t xml:space="preserve">Race, with the Asian Sub-categories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Enrolled Subjects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Race and Asian Sub-categories</t>
+  </si>
+  <si>
     <t xml:space="preserve">Systolic Blood Pressure (mmHg): Mean Change from Baseline at Week 24 (95% CI)</t>
   </si>
   <si>
@@ -1272,6 +1293,15 @@
   </si>
   <si>
     <t xml:space="preserve">SCRF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Race with its Asian sub-categories nested under Asian, one block (enrolled subjects by arm, Total; the sub-categories derived for demonstration)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Race and its Asian sub-categories, two blocks (enrolled subjects by arm, Total; the sub-categories derived for demonstration)</t>
   </si>
   <si>
     <t xml:space="preserve">Demographic characteristics</t>
@@ -1760,31 +1790,31 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="C1" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="D1" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="E1" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="F1" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="G1" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="H1" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
@@ -1798,7 +1828,7 @@
         <v>78</v>
       </c>
       <c r="B3" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
@@ -1812,189 +1842,189 @@
         <v>80</v>
       </c>
       <c r="B4" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="B5" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="B6" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="G6"/>
       <c r="H6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>100</v>
+        <v>73</v>
       </c>
       <c r="B7" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C7"/>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="G7"/>
       <c r="H7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="G9"/>
       <c r="H9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B10" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C10"/>
       <c r="D10"/>
       <c r="E10"/>
       <c r="F10" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="G10"/>
       <c r="H10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="B11" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="C11"/>
-      <c r="D11" t="s">
-        <v>136</v>
-      </c>
+      <c r="D11"/>
       <c r="E11"/>
       <c r="F11" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="G11"/>
       <c r="H11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C12"/>
-      <c r="D12" t="s">
-        <v>138</v>
-      </c>
+      <c r="D12"/>
       <c r="E12"/>
       <c r="F12" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="G12"/>
       <c r="H12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>89</v>
       </c>
       <c r="B13" t="s">
+        <v>145</v>
+      </c>
+      <c r="C13"/>
+      <c r="D13" t="s">
+        <v>146</v>
+      </c>
+      <c r="E13"/>
+      <c r="F13" t="s">
         <v>139</v>
       </c>
-      <c r="C13"/>
-      <c r="D13"/>
-      <c r="E13"/>
-      <c r="F13"/>
       <c r="G13"/>
       <c r="H13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>92</v>
       </c>
       <c r="B14" t="s">
-        <v>140</v>
-      </c>
-      <c r="C14" t="s">
-        <v>141</v>
-      </c>
-      <c r="D14"/>
+        <v>147</v>
+      </c>
+      <c r="C14"/>
+      <c r="D14" t="s">
+        <v>148</v>
+      </c>
       <c r="E14"/>
-      <c r="F14"/>
+      <c r="F14" t="s">
+        <v>139</v>
+      </c>
       <c r="G14"/>
       <c r="H14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>142</v>
-      </c>
-      <c r="C15" t="s">
-        <v>143</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="C15"/>
       <c r="D15"/>
       <c r="E15"/>
       <c r="F15"/>
@@ -2003,17 +2033,49 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>144</v>
-      </c>
-      <c r="C16"/>
+        <v>150</v>
+      </c>
+      <c r="C16" t="s">
+        <v>151</v>
+      </c>
       <c r="D16"/>
       <c r="E16"/>
       <c r="F16"/>
       <c r="G16"/>
       <c r="H16"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>152</v>
+      </c>
+      <c r="C17" t="s">
+        <v>153</v>
+      </c>
+      <c r="D17"/>
+      <c r="E17"/>
+      <c r="F17"/>
+      <c r="G17"/>
+      <c r="H17"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" t="s">
+        <v>154</v>
+      </c>
+      <c r="C18"/>
+      <c r="D18"/>
+      <c r="E18"/>
+      <c r="F18"/>
+      <c r="G18"/>
+      <c r="H18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2608,56 +2670,56 @@
         <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C11" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C12" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
         <v>88</v>
-      </c>
-      <c r="B13" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" t="s">
-        <v>89</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C14" t="s">
         <v>90</v>
@@ -2667,7 +2729,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
         <v>58</v>
@@ -2680,27 +2742,79 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D16"/>
       <c r="E16"/>
     </row>
     <row r="17">
-      <c r="A17"/>
+      <c r="A17" t="s">
+        <v>92</v>
+      </c>
       <c r="B17" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" t="s">
         <v>93</v>
-      </c>
-      <c r="C17" t="s">
-        <v>94</v>
       </c>
       <c r="D17"/>
       <c r="E17"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>92</v>
+      </c>
+      <c r="B18" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18"/>
+      <c r="E18"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C19" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19"/>
+      <c r="E19"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" t="s">
+        <v>96</v>
+      </c>
+      <c r="D20"/>
+      <c r="E20"/>
+    </row>
+    <row r="21">
+      <c r="A21"/>
+      <c r="B21" t="s">
+        <v>97</v>
+      </c>
+      <c r="C21" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21"/>
+      <c r="E21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2777,7 +2891,7 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -2788,10 +2902,10 @@
         <v>73</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3">
@@ -2799,10 +2913,10 @@
         <v>73</v>
       </c>
       <c r="B3" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C3" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4">
@@ -2810,10 +2924,10 @@
         <v>75</v>
       </c>
       <c r="B4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C4" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5">
@@ -2821,32 +2935,32 @@
         <v>75</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" t="s">
         <v>100</v>
       </c>
-      <c r="B6" t="s">
-        <v>96</v>
-      </c>
       <c r="C6" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B7" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8">
@@ -2854,10 +2968,10 @@
         <v>76</v>
       </c>
       <c r="B8" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C8" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9">
@@ -2865,32 +2979,32 @@
         <v>76</v>
       </c>
       <c r="B9" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C9" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B10" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" t="s">
         <v>103</v>
-      </c>
-      <c r="B11" t="s">
-        <v>98</v>
-      </c>
-      <c r="C11" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="12">
@@ -2898,10 +3012,10 @@
         <v>78</v>
       </c>
       <c r="B12" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C12" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13">
@@ -2909,10 +3023,10 @@
         <v>78</v>
       </c>
       <c r="B13" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C13" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14">
@@ -2920,10 +3034,10 @@
         <v>80</v>
       </c>
       <c r="B14" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15">
@@ -2931,10 +3045,10 @@
         <v>80</v>
       </c>
       <c r="B15" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C15" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16">
@@ -2942,10 +3056,10 @@
         <v>82</v>
       </c>
       <c r="B16" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C16" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="17">
@@ -2953,10 +3067,10 @@
         <v>82</v>
       </c>
       <c r="B17" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C17" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
     </row>
     <row r="18">
@@ -2964,10 +3078,10 @@
         <v>85</v>
       </c>
       <c r="B18" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C18" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19">
@@ -2975,120 +3089,164 @@
         <v>85</v>
       </c>
       <c r="B19" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C19" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>86</v>
       </c>
       <c r="B20" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C20" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>86</v>
       </c>
       <c r="B21" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C21" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>89</v>
       </c>
       <c r="B22" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C22" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>89</v>
       </c>
       <c r="B23" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C23" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>88</v>
+        <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C24" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>88</v>
+        <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C25" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C26" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B27" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C27" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>33</v>
+        <v>92</v>
       </c>
       <c r="B28" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C28" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
+        <v>92</v>
+      </c>
+      <c r="B29" t="s">
+        <v>102</v>
+      </c>
+      <c r="C29" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" t="s">
+        <v>100</v>
+      </c>
+      <c r="C30" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" t="s">
+        <v>102</v>
+      </c>
+      <c r="C31" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
         <v>33</v>
       </c>
-      <c r="B29" t="s">
-        <v>98</v>
-      </c>
-      <c r="C29" t="s">
-        <v>99</v>
+      <c r="B32" t="s">
+        <v>100</v>
+      </c>
+      <c r="C32" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" t="s">
+        <v>102</v>
+      </c>
+      <c r="C33" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -3113,7 +3271,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B2" t="s">
         <v>58</v>

</xml_diff>

<commit_message>
The sample regenerated with F-14-2-4, the forest plot from its own ARD (30/30; the other programs and RTFs byte-identical)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -888,7 +888,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -998,6 +998,12 @@
     <t xml:space="preserve">table:T-14-2-2</t>
   </si>
   <si>
+    <t xml:space="preserve">F-14-2-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">own</t>
+  </si>
+  <si>
     <t xml:space="preserve">paper_size</t>
   </si>
   <si>
@@ -1181,6 +1187,9 @@
     <t xml:space="preserve">x = censored.  Dashed line: the median (probability 0.5).  The medians are those of Table 14.2.2; the hazard ratios (Cox model) are in its ARD.</t>
   </si>
   <si>
+    <t xml:space="preserve">Hazard ratio of Xanomeline High Dose vs Placebo (Cox model, unstratified) with its 95% CI, overall and within each subgroup; the figure's own ARD.  NE = not estimable.</t>
+  </si>
+  <si>
     <t xml:space="preserve">98</t>
   </si>
   <si>
@@ -1257,6 +1266,9 @@
   </si>
   <si>
     <t xml:space="preserve">Kaplan-Meier Curves of Time to First Dermatologic Event</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hazard Ratio of Time to First Dermatologic Event by Subgroup</t>
   </si>
   <si>
     <t xml:space="preserve">spec_version</t>
@@ -1421,6 +1433,9 @@
   </si>
   <si>
     <t xml:space="preserve">KM curves of the time to first dermatologic event (designed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hazard ratio of the time to first dermatologic event by subgroup (forest plot, its own ARD)</t>
   </si>
 </sst>
 </file>
@@ -1790,31 +1805,31 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C1" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E1" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F1" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="G1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="H1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
@@ -1825,10 +1840,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
@@ -1839,180 +1854,180 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B5" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B6" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="G6"/>
       <c r="H6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C7"/>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G7"/>
       <c r="H7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B8" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B9" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G9"/>
       <c r="H9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B10" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C10"/>
       <c r="D10"/>
       <c r="E10"/>
       <c r="F10" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G10"/>
       <c r="H10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C11"/>
       <c r="D11"/>
       <c r="E11"/>
       <c r="F11" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G11"/>
       <c r="H11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C12"/>
       <c r="D12"/>
       <c r="E12"/>
       <c r="F12" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G12"/>
       <c r="H12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B13" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C13"/>
       <c r="D13" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E13"/>
       <c r="F13" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G13"/>
       <c r="H13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B14" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E14"/>
       <c r="F14" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G14"/>
       <c r="H14"/>
@@ -2022,7 +2037,7 @@
         <v>28</v>
       </c>
       <c r="B15" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C15"/>
       <c r="D15"/>
@@ -2036,10 +2051,10 @@
         <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C16" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D16"/>
       <c r="E16"/>
@@ -2052,10 +2067,10 @@
         <v>32</v>
       </c>
       <c r="B17" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C17" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D17"/>
       <c r="E17"/>
@@ -2068,7 +2083,7 @@
         <v>33</v>
       </c>
       <c r="B18" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C18"/>
       <c r="D18"/>
@@ -2076,6 +2091,20 @@
       <c r="F18"/>
       <c r="G18"/>
       <c r="H18"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" t="s">
+        <v>159</v>
+      </c>
+      <c r="C19"/>
+      <c r="D19"/>
+      <c r="E19"/>
+      <c r="F19"/>
+      <c r="G19"/>
+      <c r="H19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2270,6 +2299,32 @@
       </c>
       <c r="R6"/>
     </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7"/>
+      <c r="D7"/>
+      <c r="E7"/>
+      <c r="F7"/>
+      <c r="G7"/>
+      <c r="H7"/>
+      <c r="I7"/>
+      <c r="J7"/>
+      <c r="K7"/>
+      <c r="L7"/>
+      <c r="M7"/>
+      <c r="N7"/>
+      <c r="O7"/>
+      <c r="P7"/>
+      <c r="Q7" t="s">
+        <v>37</v>
+      </c>
+      <c r="R7"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -2287,55 +2342,55 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="J1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="L1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="M1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="N1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="O1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="P1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="Q1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="R1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2">
@@ -2344,7 +2399,7 @@
       </c>
       <c r="B2"/>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -2368,7 +2423,7 @@
       </c>
       <c r="B3"/>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -2392,7 +2447,7 @@
       </c>
       <c r="B4"/>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
@@ -2416,7 +2471,7 @@
       </c>
       <c r="B5"/>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
@@ -2434,6 +2489,30 @@
       <c r="Q5"/>
       <c r="R5"/>
     </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6"/>
+      <c r="C6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6"/>
+      <c r="E6"/>
+      <c r="F6"/>
+      <c r="G6"/>
+      <c r="H6"/>
+      <c r="I6"/>
+      <c r="J6"/>
+      <c r="K6"/>
+      <c r="L6"/>
+      <c r="M6"/>
+      <c r="N6"/>
+      <c r="O6"/>
+      <c r="P6"/>
+      <c r="Q6"/>
+      <c r="R6"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -2451,48 +2530,48 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3">
       <c r="A3"/>
       <c r="B3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D3"/>
       <c r="E3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4">
       <c r="A4"/>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -2501,33 +2580,33 @@
     <row r="5">
       <c r="A5"/>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6"/>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7"/>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E7"/>
     </row>
@@ -2548,181 +2627,181 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D8"/>
       <c r="E8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" t="s">
         <v>85</v>
-      </c>
-      <c r="B10" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" t="s">
-        <v>83</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B12" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C12" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B13" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B14" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D14"/>
       <c r="E14"/>
@@ -2732,49 +2811,49 @@
         <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D15"/>
       <c r="E15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D16"/>
       <c r="E16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B17" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C17" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D17"/>
       <c r="E17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B18" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D18"/>
       <c r="E18"/>
@@ -2784,10 +2863,10 @@
         <v>32</v>
       </c>
       <c r="B19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D19"/>
       <c r="E19"/>
@@ -2797,24 +2876,37 @@
         <v>33</v>
       </c>
       <c r="B20" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C20" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D20"/>
       <c r="E20"/>
     </row>
     <row r="21">
-      <c r="A21"/>
+      <c r="A21" t="s">
+        <v>36</v>
+      </c>
       <c r="B21" t="s">
-        <v>97</v>
+        <v>60</v>
       </c>
       <c r="C21" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D21"/>
       <c r="E21"/>
+    </row>
+    <row r="22">
+      <c r="A22"/>
+      <c r="B22" t="s">
+        <v>100</v>
+      </c>
+      <c r="C22" t="s">
+        <v>101</v>
+      </c>
+      <c r="D22"/>
+      <c r="E22"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2833,16 +2925,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -2862,16 +2954,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -2891,7 +2983,7 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -2899,244 +2991,244 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C3" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C6" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B7" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C8" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C10" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B12" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C12" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C13" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C14" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B15" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C15" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B16" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C16" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B17" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C17" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B18" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C18" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B19" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C19" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B20" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C20" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B21" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C21" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C22" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B23" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C23" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="24">
@@ -3144,10 +3236,10 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C24" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="25">
@@ -3155,10 +3247,10 @@
         <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C25" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="26">
@@ -3166,10 +3258,10 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C26" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="27">
@@ -3177,32 +3269,32 @@
         <v>30</v>
       </c>
       <c r="B27" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C27" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B28" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C28" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B29" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C29" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30">
@@ -3210,10 +3302,10 @@
         <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C30" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="31">
@@ -3221,10 +3313,10 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C31" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="32">
@@ -3232,10 +3324,10 @@
         <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C32" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="33">
@@ -3243,10 +3335,32 @@
         <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C33" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" t="s">
         <v>103</v>
+      </c>
+      <c r="C34" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" t="s">
+        <v>105</v>
+      </c>
+      <c r="C35" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -3271,10 +3385,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
F-14-2-4 has the sample's analysis set (SAF) like every report with analyses; tests know the new figure
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -2102,7 +2102,9 @@
       <c r="C19"/>
       <c r="D19"/>
       <c r="E19"/>
-      <c r="F19"/>
+      <c r="F19" t="s">
+        <v>143</v>
+      </c>
       <c r="G19"/>
       <c r="H19"/>
     </row>

</xml_diff>

<commit_message>
The sample's race tables are demographics tables, with ASIANSUB nested under Asian (T-14-1-5) or as its own block (T-14-1-6)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -1142,7 +1142,7 @@
     <t xml:space="preserve">Enrolled subjects: all subjects of ADSL, screen failures included.  Percentages of the column's subjects.</t>
   </si>
   <si>
-    <t xml:space="preserve">Asian sub-categories (Chinese, Japanese, Korean) are derived for demonstration; they are not in the source data.</t>
+    <t xml:space="preserve">Asian sub-categories (ASIANSUB: Chinese, Japanese, Korean) are derived for demonstration; they are not in the source data.  As an EDC collects them, each race has its own sub-category column.</t>
   </si>
   <si>
     <t xml:space="preserve">T-14-1-6</t>
@@ -1229,13 +1229,13 @@
     <t xml:space="preserve">All Screen Failures</t>
   </si>
   <si>
-    <t xml:space="preserve">Race, with the Asian Sub-categories</t>
+    <t xml:space="preserve">Demographic Characteristics, with the Asian Sub-categories of Race</t>
   </si>
   <si>
     <t xml:space="preserve">All Enrolled Subjects</t>
   </si>
   <si>
-    <t xml:space="preserve">Race and Asian Sub-categories</t>
+    <t xml:space="preserve">Demographic Characteristics and the Asian Sub-categories of Race</t>
   </si>
   <si>
     <t xml:space="preserve">Systolic Blood Pressure (mmHg): Mean Change from Baseline at Week 24 (95% CI)</t>
@@ -1289,61 +1289,34 @@
     <t xml:space="preserve">Study information: dictionary versions and the dates of the data (no analysis set)</t>
   </si>
   <si>
+    <t xml:space="preserve">Demographic characteristics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographic characteristics (its ARD one ard_stack call)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subject disposition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age group and sex: the ARD keeps cards' default n, N and p; the table prints n (%) and leaves the N rows out</t>
+  </si>
+  <si>
     <t xml:space="preserve">Demographic characteristics of the screen failures (an analysis set by a condition alone)</t>
   </si>
   <si>
     <t xml:space="preserve">SCRF</t>
   </si>
   <si>
-    <t xml:space="preserve">Race with its Asian sub-categories nested under Asian, one block (enrolled subjects by arm, Total; the sub-categories derived for demonstration)</t>
+    <t xml:space="preserve">Demographics, race's Asian sub-categories nested under Asian (enrolled subjects by arm, Total; ASIANSUB derived for demonstration)</t>
   </si>
   <si>
     <t xml:space="preserve">ENR</t>
   </si>
   <si>
-    <t xml:space="preserve">Race and its Asian sub-categories, two blocks (enrolled subjects by arm, Total; the sub-categories derived for demonstration)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demographic characteristics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demographic characteristics (its ARD one ard_stack call)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subject disposition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Systolic blood pressure: change from baseline at Week 24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Age group and sex: the ARD keeps cards' default n, N and p; the table prints n (%) and leaves the N rows out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Systolic blood pressure: mean change at Week 24 (95% CI), p-value; the ARD also holds the test's method and alternative as text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEAEs by SOC / PT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data &lt;- normalize_ard(ard, hierarchy = c("AEBODSYS", "AEDECOD"),
-                      overall = "Any TEAE")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Time to first dermatologic event: KM estimates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data &lt;- normalize_ard(ard)
-# row labels: the median, and the event-free probability by day (day 0 left out)
-is_time &lt;- data$variable == "time"
-data$.label[data$variable == "prob"] &lt;- "Median (95% CI)"
-data$.label[is_time] &lt;- paste("Day", as.character(data$variable_level[is_time]))
-data &lt;- data[!(is_time &amp; as.character(data$variable_level) == "0"), ]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Listing of severe treatment-emergent adverse events</t>
+    <t xml:space="preserve">Demographics, race's Asian sub-categories as a block of their own (enrolled subjects by arm, Total; ASIANSUB derived for demonstration)</t>
   </si>
   <si>
     <t xml:space="preserve">Mean change from baseline in systolic blood pressure</t>
@@ -1372,6 +1345,9 @@
   theme_tfl() + theme(legend.position = "bottom")
 tfl_check(plot)
 content &lt;- plot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Systolic blood pressure: change from baseline at Week 24</t>
   </si>
   <si>
     <t xml:space="preserve">KM plot of the time to first dermatologic event</t>
@@ -1420,7 +1396,31 @@
 content &lt;- plot</t>
   </si>
   <si>
+    <t xml:space="preserve">Time to first dermatologic event: KM estimates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data &lt;- normalize_ard(ard)
+# row labels: the median, and the event-free probability by day (day 0 left out)
+is_time &lt;- data$variable == "time"
+data$.label[data$variable == "prob"] &lt;- "Median (95% CI)"
+data$.label[is_time] &lt;- paste("Day", as.character(data$variable_level[is_time]))
+data &lt;- data[!(is_time &amp; as.character(data$variable_level) == "0"), ]</t>
+  </si>
+  <si>
     <t xml:space="preserve">KM curves of the time to first dermatologic event (designed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Systolic blood pressure: mean change at Week 24 (95% CI), p-value; the ARD also holds the test's method and alternative as text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEAEs by SOC / PT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data &lt;- normalize_ard(ard, hierarchy = c("AEBODSYS", "AEDECOD"),
+                      overall = "Any TEAE")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listing of severe treatment-emergent adverse events</t>
   </si>
 </sst>
 </file>
@@ -1839,7 +1839,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="B4" t="s">
         <v>133</v>
@@ -1855,7 +1855,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="B5" t="s">
         <v>135</v>
@@ -1864,49 +1864,49 @@
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="B6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G6"/>
       <c r="H6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="B7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C7"/>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="G7"/>
       <c r="H7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B8" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
@@ -1919,23 +1919,23 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="B9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G9"/>
       <c r="H9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="B10" t="s">
         <v>142</v>
@@ -1944,58 +1944,56 @@
       <c r="D10"/>
       <c r="E10"/>
       <c r="F10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G10"/>
       <c r="H10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>107</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
         <v>143</v>
       </c>
-      <c r="C11"/>
+      <c r="C11" t="s">
+        <v>144</v>
+      </c>
       <c r="D11"/>
       <c r="E11"/>
-      <c r="F11" t="s">
-        <v>139</v>
-      </c>
+      <c r="F11"/>
       <c r="G11"/>
       <c r="H11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C12"/>
       <c r="D12"/>
       <c r="E12"/>
       <c r="F12" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="G12"/>
       <c r="H12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>89</v>
+        <v>32</v>
       </c>
       <c r="B13" t="s">
-        <v>145</v>
-      </c>
-      <c r="C13"/>
-      <c r="D13" t="s">
         <v>146</v>
       </c>
+      <c r="C13" t="s">
+        <v>147</v>
+      </c>
+      <c r="D13"/>
       <c r="E13"/>
-      <c r="F13" t="s">
-        <v>139</v>
-      </c>
+      <c r="F13"/>
       <c r="G13"/>
       <c r="H13"/>
     </row>
@@ -2004,25 +2002,25 @@
         <v>92</v>
       </c>
       <c r="B14" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E14"/>
       <c r="F14" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="G14"/>
       <c r="H14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C15"/>
       <c r="D15"/>
@@ -2033,39 +2031,41 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="B16" t="s">
-        <v>150</v>
-      </c>
-      <c r="C16" t="s">
         <v>151</v>
       </c>
+      <c r="C16"/>
       <c r="D16"/>
       <c r="E16"/>
-      <c r="F16"/>
+      <c r="F16" t="s">
+        <v>134</v>
+      </c>
       <c r="G16"/>
       <c r="H16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>89</v>
       </c>
       <c r="B17" t="s">
         <v>152</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17"/>
+      <c r="D17" t="s">
         <v>153</v>
       </c>
-      <c r="D17"/>
       <c r="E17"/>
-      <c r="F17"/>
+      <c r="F17" t="s">
+        <v>134</v>
+      </c>
       <c r="G17"/>
       <c r="H17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B18" t="s">
         <v>154</v>

</xml_diff>

<commit_message>
Page patterns, part C: the patterns edited in a dialog (Standard and each pattern on the same form; new, rename, remove); the sample's Compact (T-14-3-1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -291,6 +291,19 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
+          <t xml:space="preserve">The page pattern the report uses: blank, Standard (the blank rows of report, page, header, footer, titles, footnotes and tokens); a name, that pattern -- the rows whose output_id is @&lt;name&gt;, which say only what differs from Standard. The report's own rows go over its pattern's.
+Example: Compact</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
           <t xml:space="preserve">A column for people, on any sheet; never read. Any other column a sheet does not read is an error (a mistyped header).</t>
         </r>
       </text>
@@ -888,7 +901,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="166">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -959,6 +972,9 @@
     <t xml:space="preserve">ard_source</t>
   </si>
   <si>
+    <t xml:space="preserve">pattern</t>
+  </si>
+  <si>
     <t xml:space="preserve">note</t>
   </si>
   <si>
@@ -1004,6 +1020,12 @@
     <t xml:space="preserve">own</t>
   </si>
   <si>
+    <t xml:space="preserve">T-14-3-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compact</t>
+  </si>
+  <si>
     <t xml:space="preserve">paper_size</t>
   </si>
   <si>
@@ -1058,6 +1080,18 @@
     <t xml:space="preserve">landscape</t>
   </si>
   <si>
+    <t xml:space="preserve">@Compact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16</t>
+  </si>
+  <si>
     <t xml:space="preserve">line</t>
   </si>
   <si>
@@ -1161,9 +1195,6 @@
   </si>
   <si>
     <t xml:space="preserve">Systolic blood pressure after 5 minutes lying down.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-3-1</t>
   </si>
   <si>
     <t xml:space="preserve">Subjects are counted once per system organ class and once per preferred term.</t>
@@ -1805,31 +1836,31 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C1" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="D1" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E1" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F1" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="G1" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="H1" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
@@ -1840,10 +1871,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
@@ -1854,125 +1885,125 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B4" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B5" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G6"/>
       <c r="H6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B7" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="C7"/>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G7"/>
       <c r="H7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B8" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B9" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="G9"/>
       <c r="H9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B10" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="C10"/>
       <c r="D10"/>
       <c r="E10"/>
       <c r="F10" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="G10"/>
       <c r="H10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B11" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="C11" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
@@ -1982,29 +2013,29 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B12" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C12"/>
       <c r="D12"/>
       <c r="E12"/>
       <c r="F12" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G12"/>
       <c r="H12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="C13" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
@@ -2014,28 +2045,28 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B14" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="E14"/>
       <c r="F14" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G14"/>
       <c r="H14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B15" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="C15"/>
       <c r="D15"/>
@@ -2046,60 +2077,60 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B16" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C16"/>
       <c r="D16"/>
       <c r="E16"/>
       <c r="F16" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G16"/>
       <c r="H16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B17" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="C17"/>
       <c r="D17"/>
       <c r="E17"/>
       <c r="F17" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G17"/>
       <c r="H17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>91</v>
+        <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="E18"/>
       <c r="F18" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G18"/>
       <c r="H18"/>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="C19"/>
       <c r="D19"/>
@@ -2174,17 +2205,20 @@
       <c r="R1" t="s">
         <v>23</v>
       </c>
+      <c r="S1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E2"/>
       <c r="F2"/>
@@ -2199,16 +2233,17 @@
       <c r="O2"/>
       <c r="P2"/>
       <c r="Q2"/>
-      <c r="R2" t="s">
-        <v>27</v>
+      <c r="R2"/>
+      <c r="S2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
@@ -2226,13 +2261,14 @@
       <c r="P3"/>
       <c r="Q3"/>
       <c r="R3"/>
+      <c r="S3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -2250,13 +2286,14 @@
       <c r="P4"/>
       <c r="Q4"/>
       <c r="R4"/>
+      <c r="S4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" t="s">
         <v>32</v>
-      </c>
-      <c r="B5" t="s">
-        <v>31</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
@@ -2274,13 +2311,14 @@
       <c r="P5"/>
       <c r="Q5"/>
       <c r="R5"/>
+      <c r="S5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
@@ -2297,16 +2335,17 @@
       <c r="O6"/>
       <c r="P6"/>
       <c r="Q6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="R6"/>
+      <c r="S6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C7"/>
       <c r="D7"/>
@@ -2323,9 +2362,35 @@
       <c r="O7"/>
       <c r="P7"/>
       <c r="Q7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="R7"/>
+      <c r="S7"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8"/>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8"/>
+      <c r="J8"/>
+      <c r="K8"/>
+      <c r="L8"/>
+      <c r="M8"/>
+      <c r="N8"/>
+      <c r="O8"/>
+      <c r="P8"/>
+      <c r="Q8"/>
+      <c r="R8" t="s">
+        <v>40</v>
+      </c>
+      <c r="S8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2344,64 +2409,64 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="H1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="I1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="L1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="M1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="N1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="O1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="P1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="Q1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="R1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B2"/>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -2421,11 +2486,11 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B3"/>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -2445,11 +2510,11 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B4"/>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
@@ -2469,11 +2534,11 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5"/>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
@@ -2493,11 +2558,11 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B6"/>
       <c r="C6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
@@ -2515,6 +2580,40 @@
       <c r="Q6"/>
       <c r="R6"/>
     </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7"/>
+      <c r="D7"/>
+      <c r="E7"/>
+      <c r="F7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G7" t="s">
+        <v>61</v>
+      </c>
+      <c r="H7" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" t="s">
+        <v>61</v>
+      </c>
+      <c r="J7"/>
+      <c r="K7"/>
+      <c r="L7"/>
+      <c r="M7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N7"/>
+      <c r="O7"/>
+      <c r="P7"/>
+      <c r="Q7"/>
+      <c r="R7"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -2532,48 +2631,48 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="E1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3">
       <c r="A3"/>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C3" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="D3"/>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4">
       <c r="A4"/>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -2582,33 +2681,33 @@
     <row r="5">
       <c r="A5"/>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6"/>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7"/>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="E7"/>
     </row>
@@ -2629,272 +2728,272 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="E1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C4" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B5" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B6" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C6" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B7" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C7" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B8" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D8"/>
       <c r="E8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B9" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C9" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B10" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B11" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C13" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>91</v>
+        <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C14" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D14"/>
       <c r="E14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C15" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D15"/>
       <c r="E15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C16" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="D16"/>
       <c r="E16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B17" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C17" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="D17"/>
       <c r="E17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B18" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C18" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D18"/>
       <c r="E18"/>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B19" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C19" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="D19"/>
       <c r="E19"/>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B20" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C20" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="D20"/>
       <c r="E20"/>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B21" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C21" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D21"/>
       <c r="E21"/>
@@ -2902,10 +3001,10 @@
     <row r="22">
       <c r="A22"/>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C22" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D22"/>
       <c r="E22"/>
@@ -2927,16 +3026,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="E1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2956,16 +3055,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="E1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2985,7 +3084,7 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -2993,376 +3092,376 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C2" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C3" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B5" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C5" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C6" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B7" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C7" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C8" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B9" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B10" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C10" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B11" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C11" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B12" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C12" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B13" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C13" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B14" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C14" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B15" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C15" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B16" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C16" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B17" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C17" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B18" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C18" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B19" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C19" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B20" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C20" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B21" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C21" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>91</v>
+        <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C22" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>91</v>
+        <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C23" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C24" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C25" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C26" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C27" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B28" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C28" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="B29" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C29" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B30" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C30" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B31" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C31" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B32" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C32" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C33" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B34" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C34" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B35" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C35" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -3387,10 +3486,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
{OUTPUT_POPULATION} by default the label of the report's analysis set; the sample's Compact on Letter (the paper says itself in a pattern's name); the pattern bar aligned
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -901,7 +901,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -1081,9 +1081,6 @@
   </si>
   <si>
     <t xml:space="preserve">@Compact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A4</t>
   </si>
   <si>
     <t xml:space="preserve">0.5</t>
@@ -1836,31 +1833,31 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C1" t="s">
         <v>134</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>135</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>136</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>137</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>138</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>139</v>
-      </c>
-      <c r="H1" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
@@ -1871,10 +1868,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
@@ -1885,112 +1882,112 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G6"/>
       <c r="H6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C7"/>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G7"/>
       <c r="H7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G9"/>
       <c r="H9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C10"/>
       <c r="D10"/>
       <c r="E10"/>
       <c r="F10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G10"/>
       <c r="H10"/>
@@ -2000,10 +1997,10 @@
         <v>31</v>
       </c>
       <c r="B11" t="s">
+        <v>152</v>
+      </c>
+      <c r="C11" t="s">
         <v>153</v>
-      </c>
-      <c r="C11" t="s">
-        <v>154</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
@@ -2013,16 +2010,16 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C12"/>
       <c r="D12"/>
       <c r="E12"/>
       <c r="F12" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G12"/>
       <c r="H12"/>
@@ -2032,10 +2029,10 @@
         <v>33</v>
       </c>
       <c r="B13" t="s">
+        <v>155</v>
+      </c>
+      <c r="C13" t="s">
         <v>156</v>
-      </c>
-      <c r="C13" t="s">
-        <v>157</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
@@ -2045,18 +2042,18 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B14" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E14"/>
       <c r="F14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G14"/>
       <c r="H14"/>
@@ -2066,7 +2063,7 @@
         <v>34</v>
       </c>
       <c r="B15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C15"/>
       <c r="D15"/>
@@ -2077,16 +2074,16 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B16" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C16"/>
       <c r="D16"/>
       <c r="E16"/>
       <c r="F16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G16"/>
       <c r="H16"/>
@@ -2096,13 +2093,13 @@
         <v>37</v>
       </c>
       <c r="B17" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C17"/>
       <c r="D17"/>
       <c r="E17"/>
       <c r="F17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G17"/>
       <c r="H17"/>
@@ -2112,15 +2109,15 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E18"/>
       <c r="F18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G18"/>
       <c r="H18"/>
@@ -2130,7 +2127,7 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C19"/>
       <c r="D19"/>
@@ -2584,29 +2581,27 @@
       <c r="A7" t="s">
         <v>59</v>
       </c>
-      <c r="B7" t="s">
-        <v>60</v>
-      </c>
+      <c r="B7"/>
       <c r="C7"/>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J7"/>
       <c r="K7"/>
       <c r="L7"/>
       <c r="M7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N7"/>
       <c r="O7"/>
@@ -2631,48 +2626,48 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" t="s">
         <v>63</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>64</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>65</v>
-      </c>
-      <c r="E1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" t="s">
         <v>67</v>
-      </c>
-      <c r="C2" t="s">
-        <v>68</v>
       </c>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3">
       <c r="A3"/>
       <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" t="s">
         <v>70</v>
-      </c>
-      <c r="C3" t="s">
-        <v>71</v>
       </c>
       <c r="D3"/>
       <c r="E3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4">
       <c r="A4"/>
       <c r="B4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -2681,33 +2676,33 @@
     <row r="5">
       <c r="A5"/>
       <c r="B5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6"/>
       <c r="B6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7"/>
       <c r="B7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E7"/>
     </row>
@@ -2728,168 +2723,168 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" t="s">
         <v>63</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>64</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>65</v>
-      </c>
-      <c r="E1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" t="s">
         <v>80</v>
-      </c>
-      <c r="C2" t="s">
-        <v>81</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" t="s">
         <v>82</v>
-      </c>
-      <c r="B3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C3" t="s">
-        <v>83</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" t="s">
         <v>85</v>
-      </c>
-      <c r="B5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C5" t="s">
-        <v>86</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" t="s">
         <v>87</v>
-      </c>
-      <c r="B6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C6" t="s">
-        <v>88</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" t="s">
         <v>89</v>
-      </c>
-      <c r="B7" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" t="s">
-        <v>90</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" t="s">
         <v>91</v>
-      </c>
-      <c r="B8" t="s">
-        <v>67</v>
-      </c>
-      <c r="C8" t="s">
-        <v>92</v>
       </c>
       <c r="D8"/>
       <c r="E8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" t="s">
         <v>95</v>
-      </c>
-      <c r="B12" t="s">
-        <v>67</v>
-      </c>
-      <c r="C12" t="s">
-        <v>96</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
@@ -2899,10 +2894,10 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D14"/>
       <c r="E14"/>
@@ -2912,49 +2907,49 @@
         <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D15"/>
       <c r="E15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D16"/>
       <c r="E16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" t="s">
         <v>100</v>
-      </c>
-      <c r="B17" t="s">
-        <v>67</v>
-      </c>
-      <c r="C17" t="s">
-        <v>101</v>
       </c>
       <c r="D17"/>
       <c r="E17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D18"/>
       <c r="E18"/>
@@ -2964,10 +2959,10 @@
         <v>33</v>
       </c>
       <c r="B19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D19"/>
       <c r="E19"/>
@@ -2977,10 +2972,10 @@
         <v>34</v>
       </c>
       <c r="B20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D20"/>
       <c r="E20"/>
@@ -2990,10 +2985,10 @@
         <v>37</v>
       </c>
       <c r="B21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D21"/>
       <c r="E21"/>
@@ -3001,10 +2996,10 @@
     <row r="22">
       <c r="A22"/>
       <c r="B22" t="s">
+        <v>105</v>
+      </c>
+      <c r="C22" t="s">
         <v>106</v>
-      </c>
-      <c r="C22" t="s">
-        <v>107</v>
       </c>
       <c r="D22"/>
       <c r="E22"/>
@@ -3026,16 +3021,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" t="s">
         <v>63</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>64</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>65</v>
-      </c>
-      <c r="E1" t="s">
-        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -3055,16 +3050,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" t="s">
         <v>63</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>64</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>65</v>
-      </c>
-      <c r="E1" t="s">
-        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -3084,7 +3079,7 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -3092,222 +3087,222 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" t="s">
         <v>109</v>
-      </c>
-      <c r="C2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" t="s">
         <v>111</v>
-      </c>
-      <c r="C3" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C4" t="s">
         <v>109</v>
-      </c>
-      <c r="C4" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" t="s">
         <v>111</v>
-      </c>
-      <c r="C5" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C6" t="s">
         <v>113</v>
-      </c>
-      <c r="B6" t="s">
-        <v>109</v>
-      </c>
-      <c r="C6" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C7" t="s">
         <v>111</v>
-      </c>
-      <c r="C7" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B9" t="s">
+        <v>110</v>
+      </c>
+      <c r="C9" t="s">
         <v>111</v>
-      </c>
-      <c r="C9" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>115</v>
+      </c>
+      <c r="B10" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" t="s">
         <v>116</v>
-      </c>
-      <c r="B10" t="s">
-        <v>109</v>
-      </c>
-      <c r="C10" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B11" t="s">
+        <v>110</v>
+      </c>
+      <c r="C11" t="s">
         <v>111</v>
-      </c>
-      <c r="C11" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B17" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C18" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B20" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B21" t="s">
+        <v>110</v>
+      </c>
+      <c r="C21" t="s">
         <v>111</v>
-      </c>
-      <c r="C21" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="22">
@@ -3315,10 +3310,10 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C22" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23">
@@ -3326,10 +3321,10 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
+        <v>110</v>
+      </c>
+      <c r="C23" t="s">
         <v>111</v>
-      </c>
-      <c r="C23" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="24">
@@ -3337,10 +3332,10 @@
         <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C24" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="25">
@@ -3348,10 +3343,10 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
+        <v>110</v>
+      </c>
+      <c r="C25" t="s">
         <v>111</v>
-      </c>
-      <c r="C25" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="26">
@@ -3359,10 +3354,10 @@
         <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C26" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27">
@@ -3370,32 +3365,32 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
+        <v>110</v>
+      </c>
+      <c r="C27" t="s">
         <v>111</v>
-      </c>
-      <c r="C27" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B28" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C28" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B29" t="s">
+        <v>110</v>
+      </c>
+      <c r="C29" t="s">
         <v>111</v>
-      </c>
-      <c r="C29" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="30">
@@ -3403,10 +3398,10 @@
         <v>33</v>
       </c>
       <c r="B30" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C30" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="31">
@@ -3414,10 +3409,10 @@
         <v>33</v>
       </c>
       <c r="B31" t="s">
+        <v>110</v>
+      </c>
+      <c r="C31" t="s">
         <v>111</v>
-      </c>
-      <c r="C31" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="32">
@@ -3425,10 +3420,10 @@
         <v>34</v>
       </c>
       <c r="B32" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C32" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="33">
@@ -3436,10 +3431,10 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
+        <v>110</v>
+      </c>
+      <c r="C33" t="s">
         <v>111</v>
-      </c>
-      <c r="C33" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="34">
@@ -3447,10 +3442,10 @@
         <v>37</v>
       </c>
       <c r="B34" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C34" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="35">
@@ -3458,10 +3453,10 @@
         <v>37</v>
       </c>
       <c r="B35" t="s">
+        <v>110</v>
+      </c>
+      <c r="C35" t="s">
         <v>111</v>
-      </c>
-      <c r="C35" t="s">
-        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -3486,10 +3481,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
A step of your own R: its rules in full, and the sample in that form
Pair B of the user-program design.  "The rules" next to the GUI | R
program switch opens the seven rules (the ja guide's chapter 11 says the
same); the code cards' tips point to them.  The sample study is made again
(data-raw/make-sample-study.R): F-14-2-1 and F-14-2-2 are figures whose
content step is R, F-14-2-2 reading T-14-2-2's ARD as `ard` (its ARD
source) instead of the ARD file, neither attaching packages; the review
has nothing to say of them.  A figure whose code reads an ARD records the
definition it was made from and is made again when it changes, as a
designed one.  The ja guide, the ja figure article and the README say
three kinds of report, each step on screen or in R.  Version 0.0.2.9206.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -83,7 +83,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">table / listing / figure / user (the report's own code leaves `content`: a data frame, rtftable pages, rtfplot figures or a list of them); blank: table.
+          <t xml:space="preserve">table / listing / figure; blank: table. A step of the report may be its own code instead (data_code, content_code).
 Example: listing</t>
         </r>
       </text>
@@ -252,7 +252,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">A figure report: the figure's width in inches (rtf_figures(width_twips = )); blank: the figure's own.
+          <t xml:space="preserve">A figure report: the figure's width in inches, drawn and placed so (rtf_figures(width_twips = )); blank: the page's body width (tfl_fig_page_size()).
 Example: 9</t>
         </r>
       </text>
@@ -265,7 +265,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">A figure report: the figure's height in inches (rtf_figures(height_twips = )); blank: the figure's own.
+          <t xml:space="preserve">A figure report: the figure's height in inches, drawn and placed so; blank: the page's body height less its title and footnote lines (tfl_fig_page_size()).
 Example: 5</t>
         </r>
       </text>
@@ -297,6 +297,32 @@
       </text>
     </comment>
     <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The report's own code for its data step, instead of the definition: R that leaves data (a table, a listing) or df (a figure); the datasets the report registers and, when it reads its ARD, ard are in reach (tfl_check_code()). Blank: the definition makes the data.
+Example: df &lt;- advs |&gt; dplyr::filter(PARAMCD == "SYSBP")</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">The report's own code for its content step, instead of the definition: R that leaves content -- a table plan, a data frame, rtftable pages, a ggplot or rtfplot figure, or a list of them -- for the report step to dress. Blank: the definition makes the content.
+Example: content &lt;- ggplot2::ggplot(df) + ggplot2::geom_line()</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -901,7 +927,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="168">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -975,6 +1001,12 @@
     <t xml:space="preserve">pattern</t>
   </si>
   <si>
+    <t xml:space="preserve">data_code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">content_code</t>
+  </si>
+  <si>
     <t xml:space="preserve">note</t>
   </si>
   <si>
@@ -999,371 +1031,10 @@
     <t xml:space="preserve">F-14-2-1</t>
   </si>
   <si>
-    <t xml:space="preserve">user</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-14-2-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-14-2-3</t>
-  </si>
-  <si>
     <t xml:space="preserve">figure</t>
   </si>
   <si>
-    <t xml:space="preserve">table:T-14-2-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F-14-2-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">own</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-3-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">paper_size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">orientation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">width_in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">height_in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">margin_top_in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">margin_bottom_in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">margin_left_in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">margin_right_in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">header_dist_in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">footer_dist_in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">font</t>
-  </si>
-  <si>
-    <t xml:space="preserve">font_size_half_points</t>
-  </si>
-  <si>
-    <t xml:space="preserve">title_format</t>
-  </si>
-  <si>
-    <t xml:space="preserve">footnote_format</t>
-  </si>
-  <si>
-    <t xml:space="preserve">title_width</t>
-  </si>
-  <si>
-    <t xml:space="preserve">footnote_width</t>
-  </si>
-  <si>
-    <t xml:space="preserve">markup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">landscape</t>
-  </si>
-  <si>
-    <t xml:space="preserve">@Compact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">line</t>
-  </si>
-  <si>
-    <t xml:space="preserve">left</t>
-  </si>
-  <si>
-    <t xml:space="preserve">center</t>
-  </si>
-  <si>
-    <t xml:space="preserve">right</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sample Pharma (tflplanner sample)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRAFT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Protocol: SAMPLE-01 (CDISC pilot data)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Page {PAGE} of {TOTAL_PAGES}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{OUTPUT_LABEL}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{OUTPUT_TITLE}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;{OUTPUT_POPULATION}&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">99</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{PROGRAM}       Generated on: {DATETIME}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-1-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SD = Standard Deviation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-1-1S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-2-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SD = Standard Deviation; SE = Standard Error; CI = Confidence Interval (t distribution).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-0-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The dictionary versions are the study's (data management plan); the dates are those of ADSL.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-1-4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SD = Standard Deviation.  Screen failures: subjects not randomized (ARM is Screen Failure).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-1-5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enrolled subjects: all subjects of ADSL, screen failures included.  Percentages of the column's subjects.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Asian sub-categories (ASIANSUB: Chinese, Japanese, Korean) are derived for demonstration; they are not in the source data.  As an EDC collects them, each race has its own sub-category column.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-1-6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-2-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CI = Confidence Interval.  95% CI and p-value: one-sample t-test of the change from baseline (H0: mean change = 0).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Systolic blood pressure after 5 minutes lying down.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subjects are counted once per system organ class and once per preferred term.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vertical bars: mean +/- SE.  Systolic blood pressure after 5 minutes lying down.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-2-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dermatologic event: first treatment-emergent skin and subcutaneous tissue disorder or application site event; censored at the end of treatment.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kaplan-Meier estimates; 95% CI of the median by the Brookmeyer-Crowley method (log transformation). NE = not estimable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">x = censored.  The number at risk is that of Table 14.2.2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">x = censored.  Dashed line: the median (probability 0.5).  The medians are those of Table 14.2.2; the hazard ratios (Cox model) are in its ARD.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hazard ratio of Xanomeline High Dose vs Placebo (Cox model, unstratified) with its 95% CI, overall and within each subgroup; the figure's own ARD.  NE = not estimable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">98</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source: CDISC pilot study ADaM data of the pharmaverseadam R package.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUTPUT_TITLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demographic Characteristics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUTPUT_POPULATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Safety Analysis Set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-1-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subject Disposition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Systolic Blood Pressure (mmHg): Change from Baseline at Week 24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-14-1-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Age Group and Sex</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Study Information</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All Subjects</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demographic Characteristics of Screen Failures</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All Screen Failures</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demographic Characteristics, with the Asian Sub-categories of Race</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All Enrolled Subjects</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demographic Characteristics and the Asian Sub-categories of Race</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Systolic Blood Pressure (mmHg): Mean Change from Baseline at Week 24 (95% CI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Treatment-Emergent Adverse Events by System Organ Class and Preferred Term</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Severe Treatment-Emergent Adverse Events</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mean (SE) Change from Baseline in Systolic Blood Pressure over Time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Time to First Dermatologic Event: Kaplan-Meier Estimates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kaplan-Meier Plot of Time to First Dermatologic Event</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kaplan-Meier Curves of Time to First Dermatologic Event</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hazard Ratio of Time to First Dermatologic Event by Subgroup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">spec_version</t>
-  </si>
-  <si>
-    <t xml:space="preserve">description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data_code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">process_code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">section</t>
-  </si>
-  <si>
-    <t xml:space="preserve">population</t>
-  </si>
-  <si>
-    <t xml:space="preserve">datasets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">batches</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(every report)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Study information: dictionary versions and the dates of the data (no analysis set)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demographic characteristics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demographic characteristics (its ARD one ard_stack call)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subject disposition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Age group and sex: the ARD keeps cards' default n, N and p; the table prints n (%) and leaves the N rows out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demographic characteristics of the screen failures (an analysis set by a condition alone)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCRF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demographics, race's Asian sub-categories nested under Asian (enrolled subjects by arm, Total; ASIANSUB derived for demonstration)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demographics, race's Asian sub-categories as a block of their own (enrolled subjects by arm, Total; ASIANSUB derived for demonstration)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mean change from baseline in systolic blood pressure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">library(ggplot2)
-saf &lt;- adsl$USUBJID[adsl$SAFFL == "Y"]
+    <t xml:space="preserve">saf &lt;- adsl$USUBJID[adsl$SAFFL == "Y"]
 d &lt;- advs[advs$PARAMCD == "SYSBP" &amp; advs$USUBJID %in% saf &amp;
             advs$AVISITN &gt; 0 &amp; !is.na(advs$CHG), ]
 m &lt;- aggregate(CHG ~ TRTA + AVISITN, data = d, FUN = function(x)
@@ -1387,23 +1058,19 @@
 content &lt;- plot</t>
   </si>
   <si>
-    <t xml:space="preserve">Systolic blood pressure: change from baseline at Week 24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KM plot of the time to first dermatologic event</t>
-  </si>
-  <si>
-    <t xml:space="preserve">library(ggplot2)
-library(ggsurvfit)
-library(patchwork)
-arms &lt;- c("Placebo", "Xanomeline Low Dose", "Xanomeline High Dose")
+    <t xml:space="preserve">F-14-2-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">table:T-14-2-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arms &lt;- c("Placebo", "Xanomeline Low Dose", "Xanomeline High Dose")
 km_df &lt;- adtte[adtte$PARAMCD == "TTDE" &amp; adtte$SAFFL == "Y", ]
 km_df$TRT01A &lt;- factor(km_df$TRT01A, levels = arms)
 km_fit &lt;- survfit2(Surv(AVAL, 1 - CNSR) ~ TRT01A, data = km_df)
-# the number at risk: the KM table's (T-14-2-2), from the study ARD --
-# checked against the curve's own count
-km_ard &lt;- readRDS(file.path(path_ard, "ard.rds"))
-risk_df &lt;- tfl_km_risk(km_ard[km_ard$output_id == "T-14-2-2", ], km_fit)
+# the number at risk: the KM table's (T-14-2-2's ARD, `ard`: the
+# figure's ARD source) -- checked against the curve's own count
+risk_df &lt;- tfl_km_risk(ard, km_fit)
 x_breaks &lt;- sort(unique(risk_df$time))
 pal &lt;- tfl_colours("treatment", arms)
 p_km &lt;- ggsurvfit(km_fit, linewidth = tfl_num("line_width", "km")) +
@@ -1434,6 +1101,369 @@
   plot_layout(heights = c(1, tfl_num("risk_height", "km")))
 tfl_check(plot)
 content &lt;- plot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-14-2-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-14-2-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">own</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-3-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">paper_size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">orientation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">width_in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">height_in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">margin_top_in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">margin_bottom_in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">margin_left_in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">margin_right_in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">header_dist_in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">footer_dist_in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">font</t>
+  </si>
+  <si>
+    <t xml:space="preserve">font_size_half_points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">title_format</t>
+  </si>
+  <si>
+    <t xml:space="preserve">footnote_format</t>
+  </si>
+  <si>
+    <t xml:space="preserve">title_width</t>
+  </si>
+  <si>
+    <t xml:space="preserve">footnote_width</t>
+  </si>
+  <si>
+    <t xml:space="preserve">markup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">landscape</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@Compact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">left</t>
+  </si>
+  <si>
+    <t xml:space="preserve">center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">right</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample Pharma (tflplanner sample)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRAFT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protocol: SAMPLE-01 (CDISC pilot data)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page {PAGE} of {TOTAL_PAGES}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{OUTPUT_LABEL}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{OUTPUT_TITLE}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;{OUTPUT_POPULATION}&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{PROGRAM}       Generated on: {DATETIME}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-1-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SD = Standard Deviation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-1-1S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-2-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SD = Standard Deviation; SE = Standard Error; CI = Confidence Interval (t distribution).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-0-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The dictionary versions are the study's (data management plan); the dates are those of ADSL.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-1-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SD = Standard Deviation.  Screen failures: subjects not randomized (ARM is Screen Failure).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-1-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enrolled subjects: all subjects of ADSL, screen failures included.  Percentages of the column's subjects.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asian sub-categories (ASIANSUB: Chinese, Japanese, Korean) are derived for demonstration; they are not in the source data.  As an EDC collects them, each race has its own sub-category column.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-1-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-2-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI = Confidence Interval.  95% CI and p-value: one-sample t-test of the change from baseline (H0: mean change = 0).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Systolic blood pressure after 5 minutes lying down.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subjects are counted once per system organ class and once per preferred term.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vertical bars: mean +/- SE.  Systolic blood pressure after 5 minutes lying down.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-2-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dermatologic event: first treatment-emergent skin and subcutaneous tissue disorder or application site event; censored at the end of treatment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaplan-Meier estimates; 95% CI of the median by the Brookmeyer-Crowley method (log transformation). NE = not estimable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x = censored.  The number at risk is that of Table 14.2.2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x = censored.  Dashed line: the median (probability 0.5).  The medians are those of Table 14.2.2; the hazard ratios (Cox model) are in its ARD.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hazard ratio of Xanomeline High Dose vs Placebo (Cox model, unstratified) with its 95% CI, overall and within each subgroup; the figure's own ARD.  NE = not estimable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: CDISC pilot study ADaM data of the pharmaverseadam R package.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUTPUT_TITLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographic Characteristics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUTPUT_POPULATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safety Analysis Set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-1-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subject Disposition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Systolic Blood Pressure (mmHg): Change from Baseline at Week 24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-14-1-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age Group and Sex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Study Information</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Subjects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographic Characteristics of Screen Failures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Screen Failures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographic Characteristics, with the Asian Sub-categories of Race</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All Enrolled Subjects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographic Characteristics and the Asian Sub-categories of Race</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Systolic Blood Pressure (mmHg): Mean Change from Baseline at Week 24 (95% CI)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Treatment-Emergent Adverse Events by System Organ Class and Preferred Term</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Severe Treatment-Emergent Adverse Events</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean (SE) Change from Baseline in Systolic Blood Pressure over Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time to First Dermatologic Event: Kaplan-Meier Estimates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaplan-Meier Plot of Time to First Dermatologic Event</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaplan-Meier Curves of Time to First Dermatologic Event</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hazard Ratio of Time to First Dermatologic Event by Subgroup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spec_version</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">setup_code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">process_code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">population</t>
+  </si>
+  <si>
+    <t xml:space="preserve">datasets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">batches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(every report)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Study information: dictionary versions and the dates of the data (no analysis set)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographic characteristics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographic characteristics (its ARD one ard_stack call)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subject disposition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age group and sex: the ARD keeps cards' default n, N and p; the table prints n (%) and leaves the N rows out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographic characteristics of the screen failures (an analysis set by a condition alone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCRF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographics, race's Asian sub-categories nested under Asian (enrolled subjects by arm, Total; ASIANSUB derived for demonstration)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demographics, race's Asian sub-categories as a block of their own (enrolled subjects by arm, Total; ASIANSUB derived for demonstration)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean change from baseline in systolic blood pressure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADSL | ADVS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Systolic blood pressure: change from baseline at Week 24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KM plot of the time to first dermatologic event</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADTTE</t>
   </si>
   <si>
     <t xml:space="preserve">Time to first dermatologic event: KM estimates</t>
@@ -1833,31 +1863,31 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C1" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="E1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="F1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="H1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C2"/>
       <c r="D2"/>
@@ -1868,10 +1898,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
@@ -1882,188 +1912,188 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G4"/>
       <c r="H4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B5" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
       <c r="E5"/>
       <c r="F5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G5"/>
       <c r="H5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B6" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G6"/>
       <c r="H6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B7" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C7"/>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G7"/>
       <c r="H7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B8" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C8"/>
       <c r="D8"/>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="G8"/>
       <c r="H8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B9" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C9"/>
       <c r="D9"/>
       <c r="E9"/>
       <c r="F9" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="G9"/>
       <c r="H9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B10" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C10"/>
       <c r="D10"/>
       <c r="E10"/>
       <c r="F10" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="G10"/>
       <c r="H10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>152</v>
-      </c>
-      <c r="C11" t="s">
-        <v>153</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="C11"/>
       <c r="D11"/>
       <c r="E11"/>
       <c r="F11"/>
-      <c r="G11"/>
+      <c r="G11" t="s">
+        <v>156</v>
+      </c>
       <c r="H11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B12" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C12"/>
       <c r="D12"/>
       <c r="E12"/>
       <c r="F12" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G12"/>
       <c r="H12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s">
-        <v>155</v>
-      </c>
-      <c r="C13" t="s">
-        <v>156</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="C13"/>
       <c r="D13"/>
       <c r="E13"/>
       <c r="F13"/>
-      <c r="G13"/>
+      <c r="G13" t="s">
+        <v>159</v>
+      </c>
       <c r="H13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B14" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C14"/>
       <c r="D14" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E14"/>
       <c r="F14" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G14"/>
       <c r="H14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C15"/>
       <c r="D15"/>
@@ -2074,60 +2104,60 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B16" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C16"/>
       <c r="D16"/>
       <c r="E16"/>
       <c r="F16" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G16"/>
       <c r="H16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C17"/>
       <c r="D17"/>
       <c r="E17"/>
       <c r="F17" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G17"/>
       <c r="H17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B18" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C18"/>
       <c r="D18" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E18"/>
       <c r="F18" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G18"/>
       <c r="H18"/>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B19" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C19"/>
       <c r="D19"/>
@@ -2205,17 +2235,23 @@
       <c r="S1" t="s">
         <v>24</v>
       </c>
+      <c r="T1" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E2"/>
       <c r="F2"/>
@@ -2231,16 +2267,18 @@
       <c r="P2"/>
       <c r="Q2"/>
       <c r="R2"/>
-      <c r="S2" t="s">
-        <v>28</v>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C3"/>
       <c r="D3"/>
@@ -2259,13 +2297,15 @@
       <c r="Q3"/>
       <c r="R3"/>
       <c r="S3"/>
+      <c r="T3"/>
+      <c r="U3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -2284,13 +2324,17 @@
       <c r="Q4"/>
       <c r="R4"/>
       <c r="S4"/>
+      <c r="T4" t="s">
+        <v>35</v>
+      </c>
+      <c r="U4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5"/>
       <c r="D5"/>
@@ -2306,16 +2350,22 @@
       <c r="N5"/>
       <c r="O5"/>
       <c r="P5"/>
-      <c r="Q5"/>
+      <c r="Q5" t="s">
+        <v>37</v>
+      </c>
       <c r="R5"/>
       <c r="S5"/>
+      <c r="T5" t="s">
+        <v>38</v>
+      </c>
+      <c r="U5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" t="s">
         <v>34</v>
-      </c>
-      <c r="B6" t="s">
-        <v>35</v>
       </c>
       <c r="C6"/>
       <c r="D6"/>
@@ -2332,17 +2382,19 @@
       <c r="O6"/>
       <c r="P6"/>
       <c r="Q6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R6"/>
       <c r="S6"/>
+      <c r="T6"/>
+      <c r="U6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7"/>
       <c r="D7"/>
@@ -2359,14 +2411,16 @@
       <c r="O7"/>
       <c r="P7"/>
       <c r="Q7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="R7"/>
       <c r="S7"/>
+      <c r="T7"/>
+      <c r="U7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2385,9 +2439,11 @@
       <c r="P8"/>
       <c r="Q8"/>
       <c r="R8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="S8"/>
+      <c r="T8"/>
+      <c r="U8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2406,64 +2462,64 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="F1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="H1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="I1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="J1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="K1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="L1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="M1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="N1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="O1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="P1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="Q1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="R1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B2"/>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
@@ -2483,11 +2539,11 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B3"/>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -2507,11 +2563,11 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B4"/>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
@@ -2531,11 +2587,11 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B5"/>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
@@ -2555,11 +2611,11 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B6"/>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
@@ -2579,29 +2635,29 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B7"/>
       <c r="C7"/>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="I7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="J7"/>
       <c r="K7"/>
       <c r="L7"/>
       <c r="M7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="N7"/>
       <c r="O7"/>
@@ -2626,48 +2682,48 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D2"/>
       <c r="E2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3">
       <c r="A3"/>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D3"/>
       <c r="E3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4">
       <c r="A4"/>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C4"/>
       <c r="D4"/>
@@ -2676,33 +2732,33 @@
     <row r="5">
       <c r="A5"/>
       <c r="B5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6"/>
       <c r="B6" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7"/>
       <c r="B7" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E7"/>
     </row>
@@ -2723,272 +2779,272 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2">
       <c r="A2"/>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D2"/>
       <c r="E2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C6" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C7" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D8"/>
       <c r="E8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B10" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C10" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D10"/>
       <c r="E10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C11" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D11"/>
       <c r="E11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C12" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D12"/>
       <c r="E12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B13" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C13" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D13"/>
       <c r="E13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C14" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D14"/>
       <c r="E14"/>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C15" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D15"/>
       <c r="E15"/>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C16" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D16"/>
       <c r="E16"/>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B17" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C17" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D17"/>
       <c r="E17"/>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B18" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C18" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D18"/>
       <c r="E18"/>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B19" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C19" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D19"/>
       <c r="E19"/>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C20" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D20"/>
       <c r="E20"/>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B21" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C21" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D21"/>
       <c r="E21"/>
@@ -2996,10 +3052,10 @@
     <row r="22">
       <c r="A22"/>
       <c r="B22" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C22" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D22"/>
       <c r="E22"/>
@@ -3021,16 +3077,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -3050,16 +3106,16 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -3079,7 +3135,7 @@
         <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -3087,376 +3143,376 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B4" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B5" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C5" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B6" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B7" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B8" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C8" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B9" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C9" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B10" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C10" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B11" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C11" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B12" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C12" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B13" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C13" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B14" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C14" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B15" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C15" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B16" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C16" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B17" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C17" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B18" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C18" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B19" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C19" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B20" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C20" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B21" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C21" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B22" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C22" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B23" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C23" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C24" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B25" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C25" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B26" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C26" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B27" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C27" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B28" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C28" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B29" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C29" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B30" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C30" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B31" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C31" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C32" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C33" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B34" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C34" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B35" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C35" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -3481,10 +3537,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
The sample's T-14-3-1 names its any-event row in tables$overall_label (#379), not in a rework line of its own
The generator writes overall_label = "Any TEAE" and no process code for
T-14-3-1; its program's normalize line is written from the definitions
(tflspec::tfl_normalize_code()) and reads the same as before.  The
starter test compares that line with the sample's.  The sample made
again: its data and the other workbooks unchanged in content.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/report_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/report_spec.xlsx
@@ -252,8 +252,8 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">A figure report: the figure's width in inches, drawn and placed so (rtf_figures(width_twips = )); blank: the page's body width (tfl_fig_page_size()).
-Example: 9</t>
+          <t xml:space="preserve">A figure report: the figure's width on the page -- a number of inches, or fit (the page's body); drawn and placed so (rtf_figures(width_twips = )). Blank: the figure's own size, as rtfreporter places it (tfl_fig_page_size()).
+Example: fit</t>
         </r>
       </text>
     </comment>
@@ -265,7 +265,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">A figure report: the figure's height in inches, drawn and placed so; blank: the page's body height less its title and footnote lines (tfl_fig_page_size()).
+          <t xml:space="preserve">A figure report: the figure's height on the page -- a number of inches, or fit (the page's body less its title and footnote lines); drawn and placed so. Blank: the figure's own size (tfl_fig_page_size()).
 Example: 5</t>
         </r>
       </text>
@@ -927,7 +927,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="167">
   <si>
     <t xml:space="preserve">key</t>
   </si>
@@ -1487,10 +1487,6 @@
   </si>
   <si>
     <t xml:space="preserve">TEAEs by SOC / PT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data &lt;- normalize_ard(ard, hierarchy = c("AEBODSYS", "AEDECOD"),
-                      overall = "Any TEAE")</t>
   </si>
   <si>
     <t xml:space="preserve">Listing of severe treatment-emergent adverse events</t>
@@ -2142,9 +2138,7 @@
         <v>165</v>
       </c>
       <c r="C18"/>
-      <c r="D18" t="s">
-        <v>166</v>
-      </c>
+      <c r="D18"/>
       <c r="E18"/>
       <c r="F18" t="s">
         <v>146</v>
@@ -2157,7 +2151,7 @@
         <v>31</v>
       </c>
       <c r="B19" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C19"/>
       <c r="D19"/>

</xml_diff>